<commit_message>
Baukosten 2.200 EUR/m2, Gastro-Ausbau 150.000 EUR, Verkauf je Partei (kein Eigenkapital), Variante B 540 m2
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJGZfxHv7bzYyqdLwg8aFJ
</commit_message>
<xml_diff>
--- a/praesentation/Rechenmodell_Baufeld3.xlsx
+++ b/praesentation/Rechenmodell_Baufeld3.xlsx
@@ -12,8 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kredit" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cashflow" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Szenarien" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variante 4 Ebenen" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hinweise" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verkauf je Partei" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variante 4 Ebenen" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hinweise" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -603,11 +604,11 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>2700</v>
+        <v>2200</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Annahme, mit Architekt prüfen</t>
+          <t>Annahme des Bauherrn (Bekanntenpreis), Angebot nötig</t>
         </is>
       </c>
     </row>
@@ -633,11 +634,11 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>310000</v>
+        <v>150000</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Küche, Bar, Möbel, Technik, Planung, Puffer</t>
+          <t>Annahme des Bauherrn, einfacher Ausbau (erste Schätzung 310.000 €)</t>
         </is>
       </c>
     </row>
@@ -2220,25 +2221,25 @@
         <v>0</v>
       </c>
       <c r="B5" s="16" t="n">
-        <v>3365481</v>
+        <v>2670731</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>12814.44</v>
+        <v>10171.81</v>
       </c>
       <c r="D5" s="21" t="n">
-        <v>1217.56</v>
+        <v>3860.19</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>15071.43</v>
+        <v>11964.38</v>
       </c>
       <c r="F5" s="21" t="n">
-        <v>-1039.43</v>
+        <v>2067.62</v>
       </c>
       <c r="G5" s="16" t="n">
-        <v>46008</v>
+        <v>37343.63</v>
       </c>
       <c r="H5" s="16" t="n">
-        <v>53407.97</v>
+        <v>43220.91</v>
       </c>
     </row>
     <row r="6">
@@ -2246,25 +2247,25 @@
         <v>0.05</v>
       </c>
       <c r="B6" s="16" t="n">
-        <v>3197206.95</v>
+        <v>2537194.45</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>12173.72</v>
+        <v>9663.219999999999</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>1858.28</v>
+        <v>4368.78</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>14317.86</v>
+        <v>11366.16</v>
       </c>
       <c r="F6" s="21" t="n">
-        <v>-285.86</v>
+        <v>2665.84</v>
       </c>
       <c r="G6" s="16" t="n">
-        <v>43907.28</v>
+        <v>35676.12</v>
       </c>
       <c r="H6" s="16" t="n">
-        <v>50937.24</v>
+        <v>41259.53</v>
       </c>
     </row>
     <row r="7">
@@ -2272,25 +2273,25 @@
         <v>0.1</v>
       </c>
       <c r="B7" s="16" t="n">
-        <v>3028932.9</v>
+        <v>2403657.9</v>
       </c>
       <c r="C7" s="16" t="n">
-        <v>11533</v>
+        <v>9154.629999999999</v>
       </c>
       <c r="D7" s="21" t="n">
-        <v>2499</v>
+        <v>4877.37</v>
       </c>
       <c r="E7" s="16" t="n">
-        <v>13564.29</v>
+        <v>10767.94</v>
       </c>
       <c r="F7" s="21" t="n">
-        <v>467.71</v>
+        <v>3264.06</v>
       </c>
       <c r="G7" s="16" t="n">
-        <v>41806.55</v>
+        <v>34008.61</v>
       </c>
       <c r="H7" s="16" t="n">
-        <v>48466.51</v>
+        <v>39298.16</v>
       </c>
     </row>
     <row r="8">
@@ -2298,25 +2299,25 @@
         <v>0.15</v>
       </c>
       <c r="B8" s="16" t="n">
-        <v>2860658.85</v>
+        <v>2270121.35</v>
       </c>
       <c r="C8" s="16" t="n">
-        <v>10892.27</v>
+        <v>8646.040000000001</v>
       </c>
       <c r="D8" s="21" t="n">
-        <v>3139.73</v>
+        <v>5385.96</v>
       </c>
       <c r="E8" s="16" t="n">
-        <v>12810.72</v>
+        <v>10169.72</v>
       </c>
       <c r="F8" s="21" t="n">
-        <v>1221.28</v>
+        <v>3862.28</v>
       </c>
       <c r="G8" s="16" t="n">
-        <v>39705.82</v>
+        <v>32341.1</v>
       </c>
       <c r="H8" s="16" t="n">
-        <v>45995.79</v>
+        <v>37336.79</v>
       </c>
     </row>
     <row r="9">
@@ -2324,25 +2325,25 @@
         <v>0.2</v>
       </c>
       <c r="B9" s="16" t="n">
-        <v>2692384.8</v>
+        <v>2136584.8</v>
       </c>
       <c r="C9" s="16" t="n">
-        <v>10251.55</v>
+        <v>8137.44</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>3780.45</v>
+        <v>5894.56</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>12057.14</v>
+        <v>9571.5</v>
       </c>
       <c r="F9" s="21" t="n">
-        <v>1974.86</v>
+        <v>4460.5</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>37605.09</v>
+        <v>30673.59</v>
       </c>
       <c r="H9" s="16" t="n">
-        <v>43525.06</v>
+        <v>35375.41</v>
       </c>
     </row>
     <row r="10">
@@ -2350,25 +2351,25 @@
         <v>0.25</v>
       </c>
       <c r="B10" s="16" t="n">
-        <v>2524110.75</v>
+        <v>2003048.25</v>
       </c>
       <c r="C10" s="16" t="n">
-        <v>9610.83</v>
+        <v>7628.85</v>
       </c>
       <c r="D10" s="21" t="n">
-        <v>4421.17</v>
+        <v>6403.15</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>11303.57</v>
+        <v>8973.280000000001</v>
       </c>
       <c r="F10" s="21" t="n">
-        <v>2728.43</v>
+        <v>5058.72</v>
       </c>
       <c r="G10" s="16" t="n">
-        <v>35504.36</v>
+        <v>29006.08</v>
       </c>
       <c r="H10" s="16" t="n">
-        <v>41054.34</v>
+        <v>33414.04</v>
       </c>
     </row>
     <row r="12">
@@ -2415,19 +2416,19 @@
         <v>0</v>
       </c>
       <c r="B14" s="21" t="n">
-        <v>-1832.44</v>
+        <v>810.1900000000001</v>
       </c>
       <c r="C14" s="21" t="n">
-        <v>-307.44</v>
+        <v>2335.19</v>
       </c>
       <c r="D14" s="21" t="n">
-        <v>1217.56</v>
+        <v>3860.19</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>2742.56</v>
+        <v>5385.19</v>
       </c>
       <c r="F14" s="21" t="n">
-        <v>4267.56</v>
+        <v>6910.19</v>
       </c>
     </row>
     <row r="15">
@@ -2435,19 +2436,19 @@
         <v>0.1</v>
       </c>
       <c r="B15" s="21" t="n">
-        <v>-551</v>
+        <v>1827.37</v>
       </c>
       <c r="C15" s="21" t="n">
-        <v>974</v>
+        <v>3352.37</v>
       </c>
       <c r="D15" s="21" t="n">
-        <v>2499</v>
+        <v>4877.37</v>
       </c>
       <c r="E15" s="21" t="n">
-        <v>4024</v>
+        <v>6402.37</v>
       </c>
       <c r="F15" s="21" t="n">
-        <v>5549</v>
+        <v>7927.37</v>
       </c>
     </row>
     <row r="16">
@@ -2455,19 +2456,19 @@
         <v>0.15</v>
       </c>
       <c r="B16" s="21" t="n">
-        <v>89.73</v>
+        <v>2335.96</v>
       </c>
       <c r="C16" s="21" t="n">
-        <v>1614.73</v>
+        <v>3860.96</v>
       </c>
       <c r="D16" s="21" t="n">
-        <v>3139.73</v>
+        <v>5385.96</v>
       </c>
       <c r="E16" s="21" t="n">
-        <v>4664.73</v>
+        <v>6910.96</v>
       </c>
       <c r="F16" s="21" t="n">
-        <v>6189.73</v>
+        <v>8435.959999999999</v>
       </c>
     </row>
     <row r="17">
@@ -2475,19 +2476,19 @@
         <v>0.2</v>
       </c>
       <c r="B17" s="21" t="n">
-        <v>730.45</v>
+        <v>2844.56</v>
       </c>
       <c r="C17" s="21" t="n">
-        <v>2255.45</v>
+        <v>4369.56</v>
       </c>
       <c r="D17" s="21" t="n">
-        <v>3780.45</v>
+        <v>5894.56</v>
       </c>
       <c r="E17" s="21" t="n">
-        <v>5305.45</v>
+        <v>7419.56</v>
       </c>
       <c r="F17" s="21" t="n">
-        <v>6830.45</v>
+        <v>8944.559999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2496,6 +2497,293 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Verkauf an die Familie: Rechnung je Partei</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Jede Partei mit eigenem Kredit ohne Eigenkapital. Preis = Selbstkosten, 3,3 % Zins, 1 % Tilgung, 10 % Rücklagen. Feste Werte aus model.js.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr"/>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>A: 1. OG 85 m²</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>A: Staffel 56 m²</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>A: Gastro (Du)</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>B: 1. OG 85 m²</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>B: Staffel 56 m²</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>B: Gastro + Büro (Du)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Preis (Selbstkosten)</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="n">
+        <v>315524.39</v>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>209194.89</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>1096573.16</v>
+      </c>
+      <c r="E5" s="16" t="n">
+        <v>297244.42</v>
+      </c>
+      <c r="F5" s="16" t="n">
+        <v>172967.47</v>
+      </c>
+      <c r="G5" s="16" t="n">
+        <v>1601252.16</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Rate pro Monat</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>1201.71</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>796.74</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>4176.43</v>
+      </c>
+      <c r="E6" s="16" t="n">
+        <v>1132.09</v>
+      </c>
+      <c r="F6" s="16" t="n">
+        <v>658.77</v>
+      </c>
+      <c r="G6" s="16" t="n">
+        <v>6098.56</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Einnahme nach Rücklagen / Gastro-Gewinn nach Lohn (+ Büro)</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>855</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>855</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>9250</v>
+      </c>
+      <c r="E7" s="16" t="n">
+        <v>855</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>855</v>
+      </c>
+      <c r="G7" s="16" t="n">
+        <v>10600</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Ergebnis pro Monat</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>-346.71</v>
+      </c>
+      <c r="C8" s="21" t="n">
+        <v>58.26</v>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>5073.57</v>
+      </c>
+      <c r="E8" s="21" t="n">
+        <v>-277.09</v>
+      </c>
+      <c r="F8" s="21" t="n">
+        <v>196.23</v>
+      </c>
+      <c r="G8" s="21" t="n">
+        <v>4501.44</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Preis für Ergebnis 0 €</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>211211.47</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>211211.47</v>
+      </c>
+      <c r="E9" s="16" t="n">
+        <v>211211.47</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>211211.47</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Lücke zum Selbstkostenpreis</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>104312.92</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>86032.95</v>
+      </c>
+      <c r="F10" s="16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Haus als Ganzes mit einem Kredit</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr"/>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>A: 340 m²</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>B: 540 m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Gesamtkosten</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="n">
+        <v>2670731</v>
+      </c>
+      <c r="C15" s="16" t="n">
+        <v>4050156</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Rate pro Monat</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="n">
+        <v>10171.81</v>
+      </c>
+      <c r="C16" s="16" t="n">
+        <v>15418.75</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Ergebnis pro Monat bei 50.000 € Umsatz</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="n">
+        <v>3860.19</v>
+      </c>
+      <c r="C17" s="21" t="n">
+        <v>2256.66</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Break-even Gastro-Umsatz</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="n">
+        <v>37343.63</v>
+      </c>
+      <c r="C18" s="16" t="n">
+        <v>42601.12</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>B: EG 540 m² (Gastro 290 + Büro 150), 1. OG 540 m², Staffel 420 m² mit 120 m² Terrasse. Nur mit Ausnahme der Stadt (Baufenster, II Vollgeschosse).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2569,10 +2857,10 @@
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>3365481</v>
+        <v>2670731</v>
       </c>
       <c r="C7" s="16" t="n">
-        <v>4421181</v>
+        <v>3530931</v>
       </c>
     </row>
     <row r="8">
@@ -2582,10 +2870,10 @@
         </is>
       </c>
       <c r="B8" s="16" t="n">
-        <v>12814.44</v>
+        <v>10171.81</v>
       </c>
       <c r="C8" s="16" t="n">
-        <v>16830.03</v>
+        <v>13443.77</v>
       </c>
     </row>
     <row r="9">
@@ -2595,10 +2883,10 @@
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>1217.56</v>
+        <v>3860.19</v>
       </c>
       <c r="C9" s="21" t="n">
-        <v>-233.03</v>
+        <v>3153.23</v>
       </c>
     </row>
     <row r="10">
@@ -2608,10 +2896,10 @@
         </is>
       </c>
       <c r="B10" s="21" t="n">
-        <v>3139.73</v>
+        <v>5385.96</v>
       </c>
       <c r="C10" s="21" t="n">
-        <v>2291.48</v>
+        <v>5169.8</v>
       </c>
     </row>
   </sheetData>
@@ -2619,7 +2907,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Variante C: 540 m2, 3 Vollgeschosse plus Holz-Penthouse (Folie, Excel, Modell)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJGZfxHv7bzYyqdLwg8aFJ
</commit_message>
<xml_diff>
--- a/praesentation/Rechenmodell_Baufeld3.xlsx
+++ b/praesentation/Rechenmodell_Baufeld3.xlsx
@@ -2502,7 +2502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -2512,6 +2512,9 @@
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2560,6 +2563,21 @@
           <t>B: Gastro + Büro (Du)</t>
         </is>
       </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>C: Regelgeschoss 85 m²</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>C: Staffel 56 m²</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>C: Gastro + Büro (Du)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -2585,6 +2603,15 @@
       <c r="G5" s="16" t="n">
         <v>1601252.16</v>
       </c>
+      <c r="H5" s="16" t="n">
+        <v>292633.16</v>
+      </c>
+      <c r="I5" s="16" t="n">
+        <v>169931.56</v>
+      </c>
+      <c r="J5" s="16" t="n">
+        <v>1578738.35</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -2610,6 +2637,15 @@
       <c r="G6" s="16" t="n">
         <v>6098.56</v>
       </c>
+      <c r="H6" s="16" t="n">
+        <v>1114.53</v>
+      </c>
+      <c r="I6" s="16" t="n">
+        <v>647.21</v>
+      </c>
+      <c r="J6" s="16" t="n">
+        <v>6012.82</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2635,6 +2671,15 @@
       <c r="G7" s="16" t="n">
         <v>10600</v>
       </c>
+      <c r="H7" s="16" t="n">
+        <v>855</v>
+      </c>
+      <c r="I7" s="16" t="n">
+        <v>855</v>
+      </c>
+      <c r="J7" s="16" t="n">
+        <v>10600</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -2660,6 +2705,15 @@
       <c r="G8" s="21" t="n">
         <v>4501.44</v>
       </c>
+      <c r="H8" s="21" t="n">
+        <v>-259.53</v>
+      </c>
+      <c r="I8" s="21" t="n">
+        <v>207.79</v>
+      </c>
+      <c r="J8" s="21" t="n">
+        <v>4587.18</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -2679,6 +2733,12 @@
       <c r="F9" s="16" t="n">
         <v>211211.47</v>
       </c>
+      <c r="H9" s="16" t="n">
+        <v>211211.47</v>
+      </c>
+      <c r="I9" s="16" t="n">
+        <v>211211.47</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -2696,6 +2756,12 @@
         <v>86032.95</v>
       </c>
       <c r="F10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="16" t="n">
+        <v>81421.69</v>
+      </c>
+      <c r="I10" s="16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2718,6 +2784,11 @@
           <t>B: 540 m²</t>
         </is>
       </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>C: 540 m², 3 Vollgeschosse + Holz-Penthouse</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -2731,6 +2802,9 @@
       <c r="C15" s="16" t="n">
         <v>4050156</v>
       </c>
+      <c r="D15" s="16" t="n">
+        <v>5416356</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -2744,6 +2818,9 @@
       <c r="C16" s="16" t="n">
         <v>15418.75</v>
       </c>
+      <c r="D16" s="16" t="n">
+        <v>20615.4</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -2757,6 +2834,9 @@
       <c r="C17" s="21" t="n">
         <v>2256.66</v>
       </c>
+      <c r="D17" s="21" t="n">
+        <v>1234.43</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -2770,11 +2850,14 @@
       <c r="C18" s="16" t="n">
         <v>42601.12</v>
       </c>
+      <c r="D18" s="16" t="n">
+        <v>45952.7</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>B: EG 540 m² (Gastro 290 + Büro 150), 1. OG 540 m², Staffel 420 m² mit 120 m² Terrasse. Nur mit Ausnahme der Stadt (Baufenster, II Vollgeschosse).</t>
+          <t>B: EG 540 m² (Gastro 290 + Büro 150), 1. OG 540 m², Staffel 420 m² mit 120 m² Terrasse. C: zusätzlich 2. OG 540 m², Höhe ca. 13 m. Nur mit Ausnahme der Stadt (Baufenster, II Vollgeschosse, 12 m).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rechnung ohne Lohn des Bauherrn
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJGZfxHv7bzYyqdLwg8aFJ
</commit_message>
<xml_diff>
--- a/praesentation/Rechenmodell_Baufeld3.xlsx
+++ b/praesentation/Rechenmodell_Baufeld3.xlsx
@@ -900,9 +900,13 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>6000</v>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>wird vorerst nicht gerechnet</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -2121,7 +2125,7 @@
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>Break-even Gastro-Umsatz (Ergebnis nach Lohn = 0)</t>
+          <t>Break-even Gastro-Umsatz (Ergebnis = 0, abzüglich Lohn aus Annahmen)</t>
         </is>
       </c>
       <c r="B15" s="15">
@@ -2227,19 +2231,19 @@
         <v>10171.81</v>
       </c>
       <c r="D5" s="21" t="n">
-        <v>3860.19</v>
+        <v>9860.190000000001</v>
       </c>
       <c r="E5" s="16" t="n">
         <v>11964.38</v>
       </c>
       <c r="F5" s="21" t="n">
-        <v>2067.62</v>
+        <v>8067.62</v>
       </c>
       <c r="G5" s="16" t="n">
-        <v>37343.63</v>
+        <v>17671.49</v>
       </c>
       <c r="H5" s="16" t="n">
-        <v>43220.91</v>
+        <v>23548.77</v>
       </c>
     </row>
     <row r="6">
@@ -2253,19 +2257,19 @@
         <v>9663.219999999999</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>4368.78</v>
+        <v>10368.78</v>
       </c>
       <c r="E6" s="16" t="n">
         <v>11366.16</v>
       </c>
       <c r="F6" s="21" t="n">
-        <v>2665.84</v>
+        <v>8665.84</v>
       </c>
       <c r="G6" s="16" t="n">
-        <v>35676.12</v>
+        <v>16003.99</v>
       </c>
       <c r="H6" s="16" t="n">
-        <v>41259.53</v>
+        <v>21587.4</v>
       </c>
     </row>
     <row r="7">
@@ -2279,19 +2283,19 @@
         <v>9154.629999999999</v>
       </c>
       <c r="D7" s="21" t="n">
-        <v>4877.37</v>
+        <v>10877.37</v>
       </c>
       <c r="E7" s="16" t="n">
         <v>10767.94</v>
       </c>
       <c r="F7" s="21" t="n">
-        <v>3264.06</v>
+        <v>9264.059999999999</v>
       </c>
       <c r="G7" s="16" t="n">
-        <v>34008.61</v>
+        <v>14336.48</v>
       </c>
       <c r="H7" s="16" t="n">
-        <v>39298.16</v>
+        <v>19626.03</v>
       </c>
     </row>
     <row r="8">
@@ -2305,19 +2309,19 @@
         <v>8646.040000000001</v>
       </c>
       <c r="D8" s="21" t="n">
-        <v>5385.96</v>
+        <v>11385.96</v>
       </c>
       <c r="E8" s="16" t="n">
         <v>10169.72</v>
       </c>
       <c r="F8" s="21" t="n">
-        <v>3862.28</v>
+        <v>9862.280000000001</v>
       </c>
       <c r="G8" s="16" t="n">
-        <v>32341.1</v>
+        <v>12668.97</v>
       </c>
       <c r="H8" s="16" t="n">
-        <v>37336.79</v>
+        <v>17664.66</v>
       </c>
     </row>
     <row r="9">
@@ -2331,19 +2335,19 @@
         <v>8137.44</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>5894.56</v>
+        <v>11894.56</v>
       </c>
       <c r="E9" s="16" t="n">
         <v>9571.5</v>
       </c>
       <c r="F9" s="21" t="n">
-        <v>4460.5</v>
+        <v>10460.5</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>30673.59</v>
+        <v>11001.46</v>
       </c>
       <c r="H9" s="16" t="n">
-        <v>35375.41</v>
+        <v>15703.28</v>
       </c>
     </row>
     <row r="10">
@@ -2357,25 +2361,25 @@
         <v>7628.85</v>
       </c>
       <c r="D10" s="21" t="n">
-        <v>6403.15</v>
+        <v>12403.15</v>
       </c>
       <c r="E10" s="16" t="n">
         <v>8973.280000000001</v>
       </c>
       <c r="F10" s="21" t="n">
-        <v>5058.72</v>
+        <v>11058.72</v>
       </c>
       <c r="G10" s="16" t="n">
-        <v>29006.08</v>
+        <v>9333.950000000001</v>
       </c>
       <c r="H10" s="16" t="n">
-        <v>33414.04</v>
+        <v>13741.91</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Ergebnis pro Monat nach Lohn, Plan 3,3 %, je Gastro-Umsatz</t>
+          <t>Ergebnis pro Monat (ohne Lohn des Bauherrn), Plan 3,3 %, je Gastro-Umsatz</t>
         </is>
       </c>
     </row>
@@ -2416,19 +2420,19 @@
         <v>0</v>
       </c>
       <c r="B14" s="21" t="n">
-        <v>810.1900000000001</v>
+        <v>6810.19</v>
       </c>
       <c r="C14" s="21" t="n">
-        <v>2335.19</v>
+        <v>8335.190000000001</v>
       </c>
       <c r="D14" s="21" t="n">
-        <v>3860.19</v>
+        <v>9860.190000000001</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>5385.19</v>
+        <v>11385.19</v>
       </c>
       <c r="F14" s="21" t="n">
-        <v>6910.19</v>
+        <v>12910.19</v>
       </c>
     </row>
     <row r="15">
@@ -2436,19 +2440,19 @@
         <v>0.1</v>
       </c>
       <c r="B15" s="21" t="n">
-        <v>1827.37</v>
+        <v>7827.37</v>
       </c>
       <c r="C15" s="21" t="n">
-        <v>3352.37</v>
+        <v>9352.370000000001</v>
       </c>
       <c r="D15" s="21" t="n">
-        <v>4877.37</v>
+        <v>10877.37</v>
       </c>
       <c r="E15" s="21" t="n">
-        <v>6402.37</v>
+        <v>12402.37</v>
       </c>
       <c r="F15" s="21" t="n">
-        <v>7927.37</v>
+        <v>13927.37</v>
       </c>
     </row>
     <row r="16">
@@ -2456,19 +2460,19 @@
         <v>0.15</v>
       </c>
       <c r="B16" s="21" t="n">
-        <v>2335.96</v>
+        <v>8335.959999999999</v>
       </c>
       <c r="C16" s="21" t="n">
-        <v>3860.96</v>
+        <v>9860.959999999999</v>
       </c>
       <c r="D16" s="21" t="n">
-        <v>5385.96</v>
+        <v>11385.96</v>
       </c>
       <c r="E16" s="21" t="n">
-        <v>6910.96</v>
+        <v>12910.96</v>
       </c>
       <c r="F16" s="21" t="n">
-        <v>8435.959999999999</v>
+        <v>14435.96</v>
       </c>
     </row>
     <row r="17">
@@ -2476,19 +2480,19 @@
         <v>0.2</v>
       </c>
       <c r="B17" s="21" t="n">
-        <v>2844.56</v>
+        <v>8844.559999999999</v>
       </c>
       <c r="C17" s="21" t="n">
-        <v>4369.56</v>
+        <v>10369.56</v>
       </c>
       <c r="D17" s="21" t="n">
-        <v>5894.56</v>
+        <v>11894.56</v>
       </c>
       <c r="E17" s="21" t="n">
-        <v>7419.56</v>
+        <v>13419.56</v>
       </c>
       <c r="F17" s="21" t="n">
-        <v>8944.559999999999</v>
+        <v>14944.56</v>
       </c>
     </row>
   </sheetData>
@@ -2650,7 +2654,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Einnahme nach Rücklagen / Gastro-Gewinn nach Lohn (+ Büro)</t>
+          <t>Einnahme nach Rücklagen / Gastro-Gewinn (+ Büro)</t>
         </is>
       </c>
       <c r="B7" s="16" t="n">
@@ -2660,7 +2664,7 @@
         <v>855</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>9250</v>
+        <v>15250</v>
       </c>
       <c r="E7" s="16" t="n">
         <v>855</v>
@@ -2669,7 +2673,7 @@
         <v>855</v>
       </c>
       <c r="G7" s="16" t="n">
-        <v>10600</v>
+        <v>16600</v>
       </c>
       <c r="H7" s="16" t="n">
         <v>855</v>
@@ -2678,7 +2682,7 @@
         <v>855</v>
       </c>
       <c r="J7" s="16" t="n">
-        <v>10600</v>
+        <v>16600</v>
       </c>
     </row>
     <row r="8">
@@ -2694,7 +2698,7 @@
         <v>58.26</v>
       </c>
       <c r="D8" s="21" t="n">
-        <v>5073.57</v>
+        <v>11073.57</v>
       </c>
       <c r="E8" s="21" t="n">
         <v>-277.09</v>
@@ -2703,7 +2707,7 @@
         <v>196.23</v>
       </c>
       <c r="G8" s="21" t="n">
-        <v>4501.44</v>
+        <v>10501.44</v>
       </c>
       <c r="H8" s="21" t="n">
         <v>-259.53</v>
@@ -2712,7 +2716,7 @@
         <v>207.79</v>
       </c>
       <c r="J8" s="21" t="n">
-        <v>4587.18</v>
+        <v>10587.18</v>
       </c>
     </row>
     <row r="9">
@@ -2829,13 +2833,13 @@
         </is>
       </c>
       <c r="B17" s="21" t="n">
-        <v>3860.19</v>
+        <v>9860.190000000001</v>
       </c>
       <c r="C17" s="21" t="n">
-        <v>2256.66</v>
+        <v>8256.66</v>
       </c>
       <c r="D17" s="21" t="n">
-        <v>1234.43</v>
+        <v>7234.43</v>
       </c>
     </row>
     <row r="18">
@@ -2845,13 +2849,13 @@
         </is>
       </c>
       <c r="B18" s="16" t="n">
-        <v>37343.63</v>
+        <v>17671.49</v>
       </c>
       <c r="C18" s="16" t="n">
-        <v>42601.12</v>
+        <v>22928.99</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>45952.7</v>
+        <v>26280.57</v>
       </c>
     </row>
     <row r="20">
@@ -2966,10 +2970,10 @@
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>3860.19</v>
+        <v>9860.190000000001</v>
       </c>
       <c r="C9" s="21" t="n">
-        <v>3153.23</v>
+        <v>9153.23</v>
       </c>
     </row>
     <row r="10">
@@ -2979,10 +2983,10 @@
         </is>
       </c>
       <c r="B10" s="21" t="n">
-        <v>5385.96</v>
+        <v>11385.96</v>
       </c>
       <c r="C10" s="21" t="n">
-        <v>5169.8</v>
+        <v>11169.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Folie und Excel: 250 EUR Plus je Wohnung (Preis, Nachlass, Ergebnis)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJGZfxHv7bzYyqdLwg8aFJ
</commit_message>
<xml_diff>
--- a/praesentation/Rechenmodell_Baufeld3.xlsx
+++ b/praesentation/Rechenmodell_Baufeld3.xlsx
@@ -2506,7 +2506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -2863,6 +2863,159 @@
         <is>
           <t>B: EG 540 m² (Gastro 290 + Büro 150), 1. OG 540 m², Staffel 420 m² mit 120 m² Terrasse. C: zusätzlich 2. OG 540 m², Höhe ca. 13 m. Nur mit Ausnahme der Stadt (Baufenster, II Vollgeschosse, 12 m).</t>
         </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>Ziel: 250 € Plus je Wohnung (Käufer ohne Eigenkapital, ohne Tilgung, Variante A)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr"/>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>1. OG 85 m²</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Staffel 56 m²</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Du</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>Zins 4,0 %: 1. OG</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>Zins 4,0 %: Staffel</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>Zins 4,0 %: Du</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Selbstkosten</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="n">
+        <v>315524.39</v>
+      </c>
+      <c r="C24" s="16" t="n">
+        <v>209194.89</v>
+      </c>
+      <c r="E24" s="16" t="n">
+        <v>315524.39</v>
+      </c>
+      <c r="F24" s="16" t="n">
+        <v>209194.89</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Verkaufspreis</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="n">
+        <v>206986</v>
+      </c>
+      <c r="C25" s="16" t="n">
+        <v>206986</v>
+      </c>
+      <c r="E25" s="16" t="n">
+        <v>168813</v>
+      </c>
+      <c r="F25" s="16" t="n">
+        <v>168813</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nachlass (von dir getragen)</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="n">
+        <v>108538.39</v>
+      </c>
+      <c r="C26" s="16" t="n">
+        <v>2208.89</v>
+      </c>
+      <c r="D26" s="16" t="n">
+        <v>332241.84</v>
+      </c>
+      <c r="E26" s="16" t="n">
+        <v>146711.39</v>
+      </c>
+      <c r="F26" s="16" t="n">
+        <v>40381.89</v>
+      </c>
+      <c r="G26" s="16" t="n">
+        <v>561279.84</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Rate pro Monat</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="n">
+        <v>605</v>
+      </c>
+      <c r="C27" s="16" t="n">
+        <v>605</v>
+      </c>
+      <c r="D27" s="16" t="n">
+        <v>5147.54</v>
+      </c>
+      <c r="E27" s="16" t="n">
+        <v>605</v>
+      </c>
+      <c r="F27" s="16" t="n">
+        <v>605</v>
+      </c>
+      <c r="G27" s="16" t="n">
+        <v>6923.99</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ergebnis pro Monat</t>
+        </is>
+      </c>
+      <c r="B28" s="21" t="n">
+        <v>250</v>
+      </c>
+      <c r="C28" s="21" t="n">
+        <v>250</v>
+      </c>
+      <c r="D28" s="21" t="n">
+        <v>10102.46</v>
+      </c>
+      <c r="E28" s="21" t="n">
+        <v>250</v>
+      </c>
+      <c r="F28" s="21" t="n">
+        <v>250</v>
+      </c>
+      <c r="G28" s="21" t="n">
+        <v>8326.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Folie 250 EUR Plus: Verkaufspreis vor Selbstkosten
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJGZfxHv7bzYyqdLwg8aFJ
</commit_message>
<xml_diff>
--- a/praesentation/Rechenmodell_Baufeld3.xlsx
+++ b/praesentation/Rechenmodell_Baufeld3.xlsx
@@ -2908,39 +2908,39 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Selbstkosten</t>
+          <t>Verkaufspreis</t>
         </is>
       </c>
       <c r="B24" s="16" t="n">
-        <v>315524.39</v>
+        <v>206986</v>
       </c>
       <c r="C24" s="16" t="n">
-        <v>209194.89</v>
+        <v>206986</v>
       </c>
       <c r="E24" s="16" t="n">
-        <v>315524.39</v>
+        <v>168813</v>
       </c>
       <c r="F24" s="16" t="n">
-        <v>209194.89</v>
+        <v>168813</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Verkaufspreis</t>
+          <t>Selbstkosten</t>
         </is>
       </c>
       <c r="B25" s="16" t="n">
-        <v>206986</v>
+        <v>315524.39</v>
       </c>
       <c r="C25" s="16" t="n">
-        <v>206986</v>
+        <v>209194.89</v>
       </c>
       <c r="E25" s="16" t="n">
-        <v>168813</v>
+        <v>315524.39</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>168813</v>
+        <v>209194.89</v>
       </c>
     </row>
     <row r="26">

</xml_diff>

<commit_message>
Verkaufsplan: Zuordnung der Wohnungen, Nebenkosten, Ablauf (Folien und Excel)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJGZfxHv7bzYyqdLwg8aFJ
</commit_message>
<xml_diff>
--- a/praesentation/Rechenmodell_Baufeld3.xlsx
+++ b/praesentation/Rechenmodell_Baufeld3.xlsx
@@ -2506,7 +2506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -3016,6 +3016,235 @@
       </c>
       <c r="G28" s="21" t="n">
         <v>8326.01</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>Verkaufsplan (Vorschlag): Preis = Selbstkosten, tilgungsfrei, 3,3 % Zins, Notar 2 %, Grunderwerbsteuer 5 % (Vater frei)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>Partei</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>Wohnung</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>Preis 15 % Förd., 2.000 €/m²</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>Notar, Steuer</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>Kredit</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>Ergebnis pro Monat</t>
+        </is>
+      </c>
+      <c r="H32" s="12" t="inlineStr">
+        <is>
+          <t>Ergebnis ohne Förderung, 2.200 €/m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Vater</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>1. OG, 85 m²</t>
+        </is>
+      </c>
+      <c r="C33" s="16" t="n">
+        <v>246039.06</v>
+      </c>
+      <c r="D33" s="16" t="n">
+        <v>4920.78</v>
+      </c>
+      <c r="E33" s="16" t="n">
+        <v>266738.03</v>
+      </c>
+      <c r="F33" s="16" t="n">
+        <v>733.53</v>
+      </c>
+      <c r="G33" s="21" t="n">
+        <v>121.47</v>
+      </c>
+      <c r="H33" s="21" t="n">
+        <v>-85.69</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Bruder</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>1. OG, 85 m²</t>
+        </is>
+      </c>
+      <c r="C34" s="16" t="n">
+        <v>246039.06</v>
+      </c>
+      <c r="D34" s="16" t="n">
+        <v>17222.73</v>
+      </c>
+      <c r="E34" s="16" t="n">
+        <v>279813.43</v>
+      </c>
+      <c r="F34" s="16" t="n">
+        <v>769.49</v>
+      </c>
+      <c r="G34" s="21" t="n">
+        <v>85.51000000000001</v>
+      </c>
+      <c r="H34" s="21" t="n">
+        <v>-131.8</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Du (eigene Wohnung)</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>1. OG, 85 m²</t>
+        </is>
+      </c>
+      <c r="C35" s="16" t="n">
+        <v>246039.06</v>
+      </c>
+      <c r="D35" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="16" t="n">
+        <v>261507.87</v>
+      </c>
+      <c r="F35" s="16" t="n">
+        <v>719.15</v>
+      </c>
+      <c r="G35" s="21" t="n">
+        <v>135.85</v>
+      </c>
+      <c r="H35" s="21" t="n">
+        <v>-67.25</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Onkel 1</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Staffel, 56 m²</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="n">
+        <v>161523.99</v>
+      </c>
+      <c r="D36" s="16" t="n">
+        <v>11306.68</v>
+      </c>
+      <c r="E36" s="16" t="n">
+        <v>183696.77</v>
+      </c>
+      <c r="F36" s="16" t="n">
+        <v>505.17</v>
+      </c>
+      <c r="G36" s="21" t="n">
+        <v>349.83</v>
+      </c>
+      <c r="H36" s="21" t="n">
+        <v>200.74</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Onkel 2</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Staffel, 56 m²</t>
+        </is>
+      </c>
+      <c r="C37" s="16" t="n">
+        <v>161523.99</v>
+      </c>
+      <c r="D37" s="16" t="n">
+        <v>11306.68</v>
+      </c>
+      <c r="E37" s="16" t="n">
+        <v>183696.77</v>
+      </c>
+      <c r="F37" s="16" t="n">
+        <v>505.17</v>
+      </c>
+      <c r="G37" s="21" t="n">
+        <v>349.83</v>
+      </c>
+      <c r="H37" s="21" t="n">
+        <v>200.74</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Onkel 3</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Staffel, 56 m²</t>
+        </is>
+      </c>
+      <c r="C38" s="16" t="n">
+        <v>161523.99</v>
+      </c>
+      <c r="D38" s="16" t="n">
+        <v>11306.68</v>
+      </c>
+      <c r="E38" s="16" t="n">
+        <v>183696.77</v>
+      </c>
+      <c r="F38" s="16" t="n">
+        <v>505.17</v>
+      </c>
+      <c r="G38" s="21" t="n">
+        <v>349.83</v>
+      </c>
+      <c r="H38" s="21" t="n">
+        <v>200.74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finale Praesentation Variante A ohne Foerderung: Verkaufsplan ohne Foerderung, Theke anthrazit, aufgeraeumt
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJGZfxHv7bzYyqdLwg8aFJ
</commit_message>
<xml_diff>
--- a/praesentation/Rechenmodell_Baufeld3.xlsx
+++ b/praesentation/Rechenmodell_Baufeld3.xlsx
@@ -2506,7 +2506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -3021,7 +3021,7 @@
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>Verkaufsplan (Vorschlag): Preis = Selbstkosten, tilgungsfrei, 3,3 % Zins, Notar 2 %, Grunderwerbsteuer 5 % (Vater frei)</t>
+          <t>Verkaufsplan (Vorschlag), ohne Förderung, 2.200 €/m², tilgungsfrei, 3,3 % Zins, Notar 2 %, Grunderwerbsteuer 5 % (Vater frei)</t>
         </is>
       </c>
     </row>
@@ -3038,32 +3038,37 @@
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>Preis 15 % Förd., 2.000 €/m²</t>
+          <t>Verkaufspreis</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
+          <t>Selbstkosten</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>Differenz (von dir getragen)</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
           <t>Notar, Steuer</t>
         </is>
       </c>
-      <c r="E32" s="12" t="inlineStr">
-        <is>
-          <t>Kredit</t>
-        </is>
-      </c>
-      <c r="F32" s="12" t="inlineStr">
-        <is>
-          <t>Rate</t>
-        </is>
-      </c>
       <c r="G32" s="12" t="inlineStr">
         <is>
+          <t>Rate (nur Zinsen)</t>
+        </is>
+      </c>
+      <c r="H32" s="12" t="inlineStr">
+        <is>
           <t>Ergebnis pro Monat</t>
         </is>
       </c>
-      <c r="H32" s="12" t="inlineStr">
-        <is>
-          <t>Ergebnis ohne Förderung, 2.200 €/m²</t>
+      <c r="I32" s="12" t="inlineStr">
+        <is>
+          <t>Ergebnis zum Selbstkostenpreis</t>
         </is>
       </c>
     </row>
@@ -3079,21 +3084,24 @@
         </is>
       </c>
       <c r="C33" s="16" t="n">
-        <v>246039.06</v>
+        <v>253240.63</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>4920.78</v>
+        <v>315524.39</v>
       </c>
       <c r="E33" s="16" t="n">
-        <v>266738.03</v>
+        <v>62283.76</v>
       </c>
       <c r="F33" s="16" t="n">
-        <v>733.53</v>
-      </c>
-      <c r="G33" s="21" t="n">
-        <v>121.47</v>
+        <v>5064.81</v>
+      </c>
+      <c r="G33" s="16" t="n">
+        <v>755</v>
       </c>
       <c r="H33" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="I33" s="21" t="n">
         <v>-85.69</v>
       </c>
     </row>
@@ -3109,21 +3117,24 @@
         </is>
       </c>
       <c r="C34" s="16" t="n">
-        <v>246039.06</v>
+        <v>241406.95</v>
       </c>
       <c r="D34" s="16" t="n">
-        <v>17222.73</v>
+        <v>315524.39</v>
       </c>
       <c r="E34" s="16" t="n">
-        <v>279813.43</v>
+        <v>74117.44</v>
       </c>
       <c r="F34" s="16" t="n">
-        <v>769.49</v>
-      </c>
-      <c r="G34" s="21" t="n">
-        <v>85.51000000000001</v>
+        <v>16898.49</v>
+      </c>
+      <c r="G34" s="16" t="n">
+        <v>755</v>
       </c>
       <c r="H34" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="I34" s="21" t="n">
         <v>-131.8</v>
       </c>
     </row>
@@ -3139,23 +3150,26 @@
         </is>
       </c>
       <c r="C35" s="16" t="n">
-        <v>246039.06</v>
+        <v>315524.39</v>
       </c>
       <c r="D35" s="16" t="n">
+        <v>315524.39</v>
+      </c>
+      <c r="E35" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="E35" s="16" t="n">
-        <v>261507.87</v>
-      </c>
       <c r="F35" s="16" t="n">
-        <v>719.15</v>
-      </c>
-      <c r="G35" s="21" t="n">
-        <v>135.85</v>
+        <v>0</v>
+      </c>
+      <c r="G35" s="16" t="n">
+        <v>922.25</v>
       </c>
       <c r="H35" s="21" t="n">
         <v>-67.25</v>
       </c>
+      <c r="I35" s="21" t="n">
+        <v>-67.25</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -3169,23 +3183,26 @@
         </is>
       </c>
       <c r="C36" s="16" t="n">
-        <v>161523.99</v>
+        <v>209194.89</v>
       </c>
       <c r="D36" s="16" t="n">
-        <v>11306.68</v>
+        <v>209194.89</v>
       </c>
       <c r="E36" s="16" t="n">
-        <v>183696.77</v>
+        <v>0</v>
       </c>
       <c r="F36" s="16" t="n">
-        <v>505.17</v>
-      </c>
-      <c r="G36" s="21" t="n">
-        <v>349.83</v>
+        <v>14643.64</v>
+      </c>
+      <c r="G36" s="16" t="n">
+        <v>654.26</v>
       </c>
       <c r="H36" s="21" t="n">
         <v>200.74</v>
       </c>
+      <c r="I36" s="21" t="n">
+        <v>200.74</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -3199,23 +3216,26 @@
         </is>
       </c>
       <c r="C37" s="16" t="n">
-        <v>161523.99</v>
+        <v>209194.89</v>
       </c>
       <c r="D37" s="16" t="n">
-        <v>11306.68</v>
+        <v>209194.89</v>
       </c>
       <c r="E37" s="16" t="n">
-        <v>183696.77</v>
+        <v>0</v>
       </c>
       <c r="F37" s="16" t="n">
-        <v>505.17</v>
-      </c>
-      <c r="G37" s="21" t="n">
-        <v>349.83</v>
+        <v>14643.64</v>
+      </c>
+      <c r="G37" s="16" t="n">
+        <v>654.26</v>
       </c>
       <c r="H37" s="21" t="n">
         <v>200.74</v>
       </c>
+      <c r="I37" s="21" t="n">
+        <v>200.74</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -3229,22 +3249,55 @@
         </is>
       </c>
       <c r="C38" s="16" t="n">
-        <v>161523.99</v>
+        <v>209194.89</v>
       </c>
       <c r="D38" s="16" t="n">
-        <v>11306.68</v>
+        <v>209194.89</v>
       </c>
       <c r="E38" s="16" t="n">
-        <v>183696.77</v>
+        <v>0</v>
       </c>
       <c r="F38" s="16" t="n">
-        <v>505.17</v>
-      </c>
-      <c r="G38" s="21" t="n">
-        <v>349.83</v>
+        <v>14643.64</v>
+      </c>
+      <c r="G38" s="16" t="n">
+        <v>654.26</v>
       </c>
       <c r="H38" s="21" t="n">
         <v>200.74</v>
+      </c>
+      <c r="I38" s="21" t="n">
+        <v>200.74</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Differenz gesamt (von dir getragen)</t>
+        </is>
+      </c>
+      <c r="C40" s="16" t="n">
+        <v>136401.2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Zinsen auf die Differenz pro Monat</t>
+        </is>
+      </c>
+      <c r="C41" s="16" t="n">
+        <v>398.69</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>Dein Ergebnis pro Monat (Gastro − Rate EG − Zinsen Differenz + eigene Wohnung)</t>
+        </is>
+      </c>
+      <c r="C42" s="21" t="n">
+        <v>10607.64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Staffelgeschoss 280 m² Holzbau, Terrasse nur 0,8 m Umlauf (58 m²), neue KI-Bilder ohne Gartenmöbel
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJGZfxHv7bzYyqdLwg8aFJ
</commit_message>
<xml_diff>
--- a/praesentation/Rechenmodell_Baufeld3.xlsx
+++ b/praesentation/Rechenmodell_Baufeld3.xlsx
@@ -589,11 +589,11 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>930</v>
+        <v>960</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>EG 340 + 1. OG 340 + Staffelgeschoss 250 (Holzbau)</t>
+          <t>EG 340 + 1. OG 340 + Staffelgeschoss 280 (Holzbau)</t>
         </is>
       </c>
     </row>
@@ -924,7 +924,7 @@
         </is>
       </c>
       <c r="B35" s="6" t="n">
-        <v>250</v>
+        <v>280</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>90</v>
+        <v>58</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
@@ -2225,25 +2225,25 @@
         <v>0</v>
       </c>
       <c r="B5" s="16" t="n">
-        <v>2670731</v>
+        <v>2716271</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>10171.81</v>
+        <v>10345.03</v>
       </c>
       <c r="D5" s="21" t="n">
-        <v>9860.190000000001</v>
+        <v>9686.969999999999</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>11964.38</v>
+        <v>12168.04</v>
       </c>
       <c r="F5" s="21" t="n">
-        <v>8067.62</v>
+        <v>7863.96</v>
       </c>
       <c r="G5" s="16" t="n">
-        <v>17671.49</v>
+        <v>18239.43</v>
       </c>
       <c r="H5" s="16" t="n">
-        <v>23548.77</v>
+        <v>24216.52</v>
       </c>
     </row>
     <row r="6">
@@ -2251,25 +2251,25 @@
         <v>0.05</v>
       </c>
       <c r="B6" s="16" t="n">
-        <v>2537194.45</v>
+        <v>2580457.45</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>9663.219999999999</v>
+        <v>9827.780000000001</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>10368.78</v>
+        <v>10204.22</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>11366.16</v>
+        <v>11559.64</v>
       </c>
       <c r="F6" s="21" t="n">
-        <v>8665.84</v>
+        <v>8472.360000000001</v>
       </c>
       <c r="G6" s="16" t="n">
-        <v>16003.99</v>
+        <v>16543.53</v>
       </c>
       <c r="H6" s="16" t="n">
-        <v>21587.4</v>
+        <v>22221.76</v>
       </c>
     </row>
     <row r="7">
@@ -2277,25 +2277,25 @@
         <v>0.1</v>
       </c>
       <c r="B7" s="16" t="n">
-        <v>2403657.9</v>
+        <v>2444643.9</v>
       </c>
       <c r="C7" s="16" t="n">
-        <v>9154.629999999999</v>
+        <v>9310.52</v>
       </c>
       <c r="D7" s="21" t="n">
-        <v>10877.37</v>
+        <v>10721.48</v>
       </c>
       <c r="E7" s="16" t="n">
-        <v>10767.94</v>
+        <v>10951.24</v>
       </c>
       <c r="F7" s="21" t="n">
-        <v>9264.059999999999</v>
+        <v>9080.76</v>
       </c>
       <c r="G7" s="16" t="n">
-        <v>14336.48</v>
+        <v>14847.62</v>
       </c>
       <c r="H7" s="16" t="n">
-        <v>19626.03</v>
+        <v>20227</v>
       </c>
     </row>
     <row r="8">
@@ -2303,25 +2303,25 @@
         <v>0.15</v>
       </c>
       <c r="B8" s="16" t="n">
-        <v>2270121.35</v>
+        <v>2308830.35</v>
       </c>
       <c r="C8" s="16" t="n">
-        <v>8646.040000000001</v>
+        <v>8793.27</v>
       </c>
       <c r="D8" s="21" t="n">
-        <v>11385.96</v>
+        <v>11238.73</v>
       </c>
       <c r="E8" s="16" t="n">
-        <v>10169.72</v>
+        <v>10342.83</v>
       </c>
       <c r="F8" s="21" t="n">
-        <v>9862.280000000001</v>
+        <v>9689.17</v>
       </c>
       <c r="G8" s="16" t="n">
-        <v>12668.97</v>
+        <v>13151.72</v>
       </c>
       <c r="H8" s="16" t="n">
-        <v>17664.66</v>
+        <v>18232.24</v>
       </c>
     </row>
     <row r="9">
@@ -2329,25 +2329,25 @@
         <v>0.2</v>
       </c>
       <c r="B9" s="16" t="n">
-        <v>2136584.8</v>
+        <v>2173016.8</v>
       </c>
       <c r="C9" s="16" t="n">
-        <v>8137.44</v>
+        <v>8276.02</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>11894.56</v>
+        <v>11755.98</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>9571.5</v>
+        <v>9734.43</v>
       </c>
       <c r="F9" s="21" t="n">
-        <v>10460.5</v>
+        <v>10297.57</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>11001.46</v>
+        <v>11455.81</v>
       </c>
       <c r="H9" s="16" t="n">
-        <v>15703.28</v>
+        <v>16237.48</v>
       </c>
     </row>
     <row r="10">
@@ -2355,25 +2355,25 @@
         <v>0.25</v>
       </c>
       <c r="B10" s="16" t="n">
-        <v>2003048.25</v>
+        <v>2037203.25</v>
       </c>
       <c r="C10" s="16" t="n">
-        <v>7628.85</v>
+        <v>7758.77</v>
       </c>
       <c r="D10" s="21" t="n">
-        <v>12403.15</v>
+        <v>12273.23</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>8973.280000000001</v>
+        <v>9126.030000000001</v>
       </c>
       <c r="F10" s="21" t="n">
-        <v>11058.72</v>
+        <v>10905.97</v>
       </c>
       <c r="G10" s="16" t="n">
-        <v>9333.950000000001</v>
+        <v>9759.9</v>
       </c>
       <c r="H10" s="16" t="n">
-        <v>13741.91</v>
+        <v>14242.72</v>
       </c>
     </row>
     <row r="12">
@@ -2420,19 +2420,19 @@
         <v>0</v>
       </c>
       <c r="B14" s="21" t="n">
-        <v>6810.19</v>
+        <v>6636.97</v>
       </c>
       <c r="C14" s="21" t="n">
-        <v>8335.190000000001</v>
+        <v>8161.97</v>
       </c>
       <c r="D14" s="21" t="n">
-        <v>9860.190000000001</v>
+        <v>9686.969999999999</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>11385.19</v>
+        <v>11211.97</v>
       </c>
       <c r="F14" s="21" t="n">
-        <v>12910.19</v>
+        <v>12736.97</v>
       </c>
     </row>
     <row r="15">
@@ -2440,19 +2440,19 @@
         <v>0.1</v>
       </c>
       <c r="B15" s="21" t="n">
-        <v>7827.37</v>
+        <v>7671.48</v>
       </c>
       <c r="C15" s="21" t="n">
-        <v>9352.370000000001</v>
+        <v>9196.48</v>
       </c>
       <c r="D15" s="21" t="n">
-        <v>10877.37</v>
+        <v>10721.48</v>
       </c>
       <c r="E15" s="21" t="n">
-        <v>12402.37</v>
+        <v>12246.48</v>
       </c>
       <c r="F15" s="21" t="n">
-        <v>13927.37</v>
+        <v>13771.48</v>
       </c>
     </row>
     <row r="16">
@@ -2460,19 +2460,19 @@
         <v>0.15</v>
       </c>
       <c r="B16" s="21" t="n">
-        <v>8335.959999999999</v>
+        <v>8188.73</v>
       </c>
       <c r="C16" s="21" t="n">
-        <v>9860.959999999999</v>
+        <v>9713.73</v>
       </c>
       <c r="D16" s="21" t="n">
-        <v>11385.96</v>
+        <v>11238.73</v>
       </c>
       <c r="E16" s="21" t="n">
-        <v>12910.96</v>
+        <v>12763.73</v>
       </c>
       <c r="F16" s="21" t="n">
-        <v>14435.96</v>
+        <v>14288.73</v>
       </c>
     </row>
     <row r="17">
@@ -2480,19 +2480,19 @@
         <v>0.2</v>
       </c>
       <c r="B17" s="21" t="n">
-        <v>8844.559999999999</v>
+        <v>8705.98</v>
       </c>
       <c r="C17" s="21" t="n">
-        <v>10369.56</v>
+        <v>10230.98</v>
       </c>
       <c r="D17" s="21" t="n">
-        <v>11894.56</v>
+        <v>11755.98</v>
       </c>
       <c r="E17" s="21" t="n">
-        <v>13419.56</v>
+        <v>13280.98</v>
       </c>
       <c r="F17" s="21" t="n">
-        <v>14944.56</v>
+        <v>14805.98</v>
       </c>
     </row>
   </sheetData>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="C4" s="12" t="inlineStr">
         <is>
-          <t>A: Staffel 56 m²</t>
+          <t>A: Staffel 63 m²</t>
         </is>
       </c>
       <c r="D4" s="12" t="inlineStr">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="F4" s="12" t="inlineStr">
         <is>
-          <t>B: Staffel 56 m²</t>
+          <t>B: Staffel 63 m²</t>
         </is>
       </c>
       <c r="G4" s="12" t="inlineStr">
@@ -2574,7 +2574,7 @@
       </c>
       <c r="I4" s="12" t="inlineStr">
         <is>
-          <t>C: Staffel 56 m²</t>
+          <t>C: Staffel 63 m²</t>
         </is>
       </c>
       <c r="J4" s="12" t="inlineStr">
@@ -2590,31 +2590,31 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>315524.39</v>
+        <v>314624.67</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>209194.89</v>
+        <v>226174.33</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>1096573.16</v>
+        <v>1093874</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>297244.42</v>
+        <v>296791.94</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>172967.47</v>
+        <v>216266.8</v>
       </c>
       <c r="G5" s="16" t="n">
-        <v>1601252.16</v>
+        <v>1599043.01</v>
       </c>
       <c r="H5" s="16" t="n">
-        <v>292633.16</v>
+        <v>292386.83</v>
       </c>
       <c r="I5" s="16" t="n">
-        <v>169931.56</v>
+        <v>212543.49</v>
       </c>
       <c r="J5" s="16" t="n">
-        <v>1578738.35</v>
+        <v>1577535.69</v>
       </c>
     </row>
     <row r="6">
@@ -2624,31 +2624,31 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>1201.71</v>
+        <v>1198.26</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>796.74</v>
+        <v>861.39</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>4176.43</v>
+        <v>4166.06</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>1132.09</v>
+        <v>1130.34</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>658.77</v>
+        <v>823.66</v>
       </c>
       <c r="G6" s="16" t="n">
-        <v>6098.56</v>
+        <v>6090.02</v>
       </c>
       <c r="H6" s="16" t="n">
-        <v>1114.53</v>
+        <v>1113.57</v>
       </c>
       <c r="I6" s="16" t="n">
-        <v>647.21</v>
+        <v>809.48</v>
       </c>
       <c r="J6" s="16" t="n">
-        <v>6012.82</v>
+        <v>6008.11</v>
       </c>
     </row>
     <row r="7">
@@ -2692,31 +2692,31 @@
         </is>
       </c>
       <c r="B8" s="21" t="n">
-        <v>-346.71</v>
+        <v>-343.26</v>
       </c>
       <c r="C8" s="21" t="n">
-        <v>58.26</v>
+        <v>-6.39</v>
       </c>
       <c r="D8" s="21" t="n">
-        <v>11073.57</v>
+        <v>11083.94</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>-277.09</v>
+        <v>-275.34</v>
       </c>
       <c r="F8" s="21" t="n">
-        <v>196.23</v>
+        <v>31.34</v>
       </c>
       <c r="G8" s="21" t="n">
-        <v>10501.44</v>
+        <v>10509.98</v>
       </c>
       <c r="H8" s="21" t="n">
-        <v>-259.53</v>
+        <v>-258.57</v>
       </c>
       <c r="I8" s="21" t="n">
-        <v>207.79</v>
+        <v>45.52</v>
       </c>
       <c r="J8" s="21" t="n">
-        <v>10587.18</v>
+        <v>10591.89</v>
       </c>
     </row>
     <row r="9">
@@ -2726,22 +2726,22 @@
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>211211.47</v>
+        <v>211220.58</v>
       </c>
       <c r="C9" s="16" t="n">
-        <v>211211.47</v>
+        <v>211220.58</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>211211.47</v>
+        <v>211220.58</v>
       </c>
       <c r="F9" s="16" t="n">
-        <v>211211.47</v>
+        <v>211220.58</v>
       </c>
       <c r="H9" s="16" t="n">
-        <v>211211.47</v>
+        <v>211220.58</v>
       </c>
       <c r="I9" s="16" t="n">
-        <v>211211.47</v>
+        <v>211220.58</v>
       </c>
     </row>
     <row r="10">
@@ -2751,22 +2751,22 @@
         </is>
       </c>
       <c r="B10" s="16" t="n">
-        <v>104312.92</v>
+        <v>103404.09</v>
       </c>
       <c r="C10" s="16" t="n">
-        <v>0</v>
+        <v>14953.75</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>86032.95</v>
+        <v>85571.36</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>0</v>
+        <v>5046.22</v>
       </c>
       <c r="H10" s="16" t="n">
-        <v>81421.69</v>
+        <v>81166.25</v>
       </c>
       <c r="I10" s="16" t="n">
-        <v>0</v>
+        <v>1322.91</v>
       </c>
     </row>
     <row r="13">
@@ -2801,13 +2801,13 @@
         </is>
       </c>
       <c r="B15" s="16" t="n">
-        <v>2670731</v>
+        <v>2716271</v>
       </c>
       <c r="C15" s="16" t="n">
-        <v>4050156</v>
+        <v>4112256</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>5416356</v>
+        <v>5478456</v>
       </c>
     </row>
     <row r="16">
@@ -2817,13 +2817,13 @@
         </is>
       </c>
       <c r="B16" s="16" t="n">
-        <v>10171.81</v>
+        <v>10345.03</v>
       </c>
       <c r="C16" s="16" t="n">
-        <v>15418.75</v>
+        <v>15654.96</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>20615.4</v>
+        <v>20851.61</v>
       </c>
     </row>
     <row r="17">
@@ -2833,13 +2833,13 @@
         </is>
       </c>
       <c r="B17" s="21" t="n">
-        <v>9860.190000000001</v>
+        <v>9686.969999999999</v>
       </c>
       <c r="C17" s="21" t="n">
-        <v>8256.66</v>
+        <v>7889.68</v>
       </c>
       <c r="D17" s="21" t="n">
-        <v>7234.43</v>
+        <v>6867.45</v>
       </c>
     </row>
     <row r="18">
@@ -2849,13 +2849,13 @@
         </is>
       </c>
       <c r="B18" s="16" t="n">
-        <v>17671.49</v>
+        <v>18239.43</v>
       </c>
       <c r="C18" s="16" t="n">
-        <v>22928.99</v>
+        <v>24132.19</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>26280.57</v>
+        <v>27483.77</v>
       </c>
     </row>
     <row r="20">
@@ -2881,7 +2881,7 @@
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>Staffel 56 m²</t>
+          <t>Staffel 63 m²</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -2912,16 +2912,16 @@
         </is>
       </c>
       <c r="B24" s="16" t="n">
-        <v>206986</v>
+        <v>206991</v>
       </c>
       <c r="C24" s="16" t="n">
-        <v>206986</v>
+        <v>206991</v>
       </c>
       <c r="E24" s="16" t="n">
-        <v>168813</v>
+        <v>168818</v>
       </c>
       <c r="F24" s="16" t="n">
-        <v>168813</v>
+        <v>168818</v>
       </c>
     </row>
     <row r="25">
@@ -2931,16 +2931,16 @@
         </is>
       </c>
       <c r="B25" s="16" t="n">
-        <v>315524.39</v>
+        <v>314624.67</v>
       </c>
       <c r="C25" s="16" t="n">
-        <v>209194.89</v>
+        <v>226174.33</v>
       </c>
       <c r="E25" s="16" t="n">
-        <v>315524.39</v>
+        <v>314624.67</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>209194.89</v>
+        <v>226174.33</v>
       </c>
     </row>
     <row r="26">
@@ -2950,22 +2950,22 @@
         </is>
       </c>
       <c r="B26" s="16" t="n">
-        <v>108538.39</v>
+        <v>107633.67</v>
       </c>
       <c r="C26" s="16" t="n">
-        <v>2208.89</v>
+        <v>19183.33</v>
       </c>
       <c r="D26" s="16" t="n">
-        <v>332241.84</v>
+        <v>380451</v>
       </c>
       <c r="E26" s="16" t="n">
-        <v>146711.39</v>
+        <v>145806.67</v>
       </c>
       <c r="F26" s="16" t="n">
-        <v>40381.89</v>
+        <v>57356.33</v>
       </c>
       <c r="G26" s="16" t="n">
-        <v>561279.84</v>
+        <v>609489</v>
       </c>
     </row>
     <row r="27">
@@ -2981,7 +2981,7 @@
         <v>605</v>
       </c>
       <c r="D27" s="16" t="n">
-        <v>5147.54</v>
+        <v>5278.06</v>
       </c>
       <c r="E27" s="16" t="n">
         <v>605</v>
@@ -2990,7 +2990,7 @@
         <v>605</v>
       </c>
       <c r="G27" s="16" t="n">
-        <v>6923.99</v>
+        <v>7084.47</v>
       </c>
     </row>
     <row r="28">
@@ -3006,7 +3006,7 @@
         <v>250</v>
       </c>
       <c r="D28" s="21" t="n">
-        <v>10102.46</v>
+        <v>9971.940000000001</v>
       </c>
       <c r="E28" s="21" t="n">
         <v>250</v>
@@ -3015,7 +3015,7 @@
         <v>250</v>
       </c>
       <c r="G28" s="21" t="n">
-        <v>8326.01</v>
+        <v>8165.53</v>
       </c>
     </row>
     <row r="31">
@@ -3084,16 +3084,16 @@
         </is>
       </c>
       <c r="C33" s="16" t="n">
-        <v>253240.63</v>
+        <v>253246.09</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>315524.39</v>
+        <v>314624.67</v>
       </c>
       <c r="E33" s="16" t="n">
-        <v>62283.76</v>
+        <v>61378.58</v>
       </c>
       <c r="F33" s="16" t="n">
-        <v>5064.81</v>
+        <v>5064.92</v>
       </c>
       <c r="G33" s="16" t="n">
         <v>755</v>
@@ -3102,7 +3102,7 @@
         <v>100</v>
       </c>
       <c r="I33" s="21" t="n">
-        <v>-85.69</v>
+        <v>-82.98999999999999</v>
       </c>
     </row>
     <row r="34">
@@ -3117,16 +3117,16 @@
         </is>
       </c>
       <c r="C34" s="16" t="n">
-        <v>241406.95</v>
+        <v>241412.16</v>
       </c>
       <c r="D34" s="16" t="n">
-        <v>315524.39</v>
+        <v>314624.67</v>
       </c>
       <c r="E34" s="16" t="n">
-        <v>74117.44</v>
+        <v>73212.50999999999</v>
       </c>
       <c r="F34" s="16" t="n">
-        <v>16898.49</v>
+        <v>16898.85</v>
       </c>
       <c r="G34" s="16" t="n">
         <v>755</v>
@@ -3135,7 +3135,7 @@
         <v>100</v>
       </c>
       <c r="I34" s="21" t="n">
-        <v>-131.8</v>
+        <v>-128.97</v>
       </c>
     </row>
     <row r="35">
@@ -3150,10 +3150,10 @@
         </is>
       </c>
       <c r="C35" s="16" t="n">
-        <v>315524.39</v>
+        <v>314624.67</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>315524.39</v>
+        <v>314624.67</v>
       </c>
       <c r="E35" s="16" t="n">
         <v>0</v>
@@ -3162,13 +3162,13 @@
         <v>0</v>
       </c>
       <c r="G35" s="16" t="n">
-        <v>922.25</v>
+        <v>919.6</v>
       </c>
       <c r="H35" s="21" t="n">
-        <v>-67.25</v>
+        <v>-64.59999999999999</v>
       </c>
       <c r="I35" s="21" t="n">
-        <v>-67.25</v>
+        <v>-64.59999999999999</v>
       </c>
     </row>
     <row r="36">
@@ -3179,29 +3179,29 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Staffel, 56 m²</t>
+          <t>Staffel, 63 m²</t>
         </is>
       </c>
       <c r="C36" s="16" t="n">
-        <v>209194.89</v>
+        <v>226174.33</v>
       </c>
       <c r="D36" s="16" t="n">
-        <v>209194.89</v>
+        <v>226174.33</v>
       </c>
       <c r="E36" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="16" t="n">
-        <v>14643.64</v>
+        <v>15832.2</v>
       </c>
       <c r="G36" s="16" t="n">
-        <v>654.26</v>
+        <v>707.34</v>
       </c>
       <c r="H36" s="21" t="n">
-        <v>200.74</v>
+        <v>147.66</v>
       </c>
       <c r="I36" s="21" t="n">
-        <v>200.74</v>
+        <v>147.66</v>
       </c>
     </row>
     <row r="37">
@@ -3212,29 +3212,29 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Staffel, 56 m²</t>
+          <t>Staffel, 63 m²</t>
         </is>
       </c>
       <c r="C37" s="16" t="n">
-        <v>209194.89</v>
+        <v>226174.33</v>
       </c>
       <c r="D37" s="16" t="n">
-        <v>209194.89</v>
+        <v>226174.33</v>
       </c>
       <c r="E37" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="16" t="n">
-        <v>14643.64</v>
+        <v>15832.2</v>
       </c>
       <c r="G37" s="16" t="n">
-        <v>654.26</v>
+        <v>707.34</v>
       </c>
       <c r="H37" s="21" t="n">
-        <v>200.74</v>
+        <v>147.66</v>
       </c>
       <c r="I37" s="21" t="n">
-        <v>200.74</v>
+        <v>147.66</v>
       </c>
     </row>
     <row r="38">
@@ -3245,29 +3245,29 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Staffel, 56 m²</t>
+          <t>Staffel, 63 m²</t>
         </is>
       </c>
       <c r="C38" s="16" t="n">
-        <v>209194.89</v>
+        <v>226174.33</v>
       </c>
       <c r="D38" s="16" t="n">
-        <v>209194.89</v>
+        <v>226174.33</v>
       </c>
       <c r="E38" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F38" s="16" t="n">
-        <v>14643.64</v>
+        <v>15832.2</v>
       </c>
       <c r="G38" s="16" t="n">
-        <v>654.26</v>
+        <v>707.34</v>
       </c>
       <c r="H38" s="21" t="n">
-        <v>200.74</v>
+        <v>147.66</v>
       </c>
       <c r="I38" s="21" t="n">
-        <v>200.74</v>
+        <v>147.66</v>
       </c>
     </row>
     <row r="40">
@@ -3277,7 +3277,7 @@
         </is>
       </c>
       <c r="C40" s="16" t="n">
-        <v>136401.2</v>
+        <v>134591.08</v>
       </c>
     </row>
     <row r="41">
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="C41" s="16" t="n">
-        <v>398.69</v>
+        <v>393.39</v>
       </c>
     </row>
     <row r="42">
@@ -3297,7 +3297,7 @@
         </is>
       </c>
       <c r="C42" s="21" t="n">
-        <v>10607.64</v>
+        <v>10625.95</v>
       </c>
     </row>
   </sheetData>
@@ -3366,10 +3366,10 @@
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>930</v>
+        <v>960</v>
       </c>
       <c r="C6" s="23" t="n">
-        <v>1270</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="7">
@@ -3379,10 +3379,10 @@
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>2670731</v>
+        <v>2716271</v>
       </c>
       <c r="C7" s="16" t="n">
-        <v>3530931</v>
+        <v>3576471</v>
       </c>
     </row>
     <row r="8">
@@ -3392,10 +3392,10 @@
         </is>
       </c>
       <c r="B8" s="16" t="n">
-        <v>10171.81</v>
+        <v>10345.03</v>
       </c>
       <c r="C8" s="16" t="n">
-        <v>13443.77</v>
+        <v>13616.99</v>
       </c>
     </row>
     <row r="9">
@@ -3405,10 +3405,10 @@
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>9860.190000000001</v>
+        <v>9686.969999999999</v>
       </c>
       <c r="C9" s="21" t="n">
-        <v>9153.23</v>
+        <v>8980.01</v>
       </c>
     </row>
     <row r="10">
@@ -3418,10 +3418,10 @@
         </is>
       </c>
       <c r="B10" s="21" t="n">
-        <v>11385.96</v>
+        <v>11238.73</v>
       </c>
       <c r="C10" s="21" t="n">
-        <v>11169.8</v>
+        <v>11022.56</v>
       </c>
     </row>
   </sheetData>
@@ -3486,7 +3486,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>• Staffelgeschoss (ca. 250 m², Holzbau, Terrasse rundum) und Gesamthöhe ca. 9,90 m müssen mit der Stadt abgestimmt werden.</t>
+          <t>• Staffelgeschoss (ca. 280 m², Holzbau, schmale Terrasse rundum) und Gesamthöhe ca. 9,90 m müssen mit der Stadt abgestimmt werden.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hauptvariante B: 540 m² Grundfläche, 8 Wohnungen, Büro im EG; neue einheitliche KI-Bilder zur Werlter Mitte
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJGZfxHv7bzYyqdLwg8aFJ
</commit_message>
<xml_diff>
--- a/praesentation/Rechenmodell_Baufeld3.xlsx
+++ b/praesentation/Rechenmodell_Baufeld3.xlsx
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -111,6 +111,7 @@
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
@@ -495,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -589,11 +590,11 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>960</v>
+        <v>1540</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>EG 340 + 1. OG 340 + Staffelgeschoss 280 (Holzbau)</t>
+          <t>EG 540 + 1. OG 540 + Staffelgeschoss 460 (Holzbau)</t>
         </is>
       </c>
     </row>
@@ -795,30 +796,31 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Anzahl Wohnungen</t>
-        </is>
-      </c>
-      <c r="B25" s="10" t="n">
-        <v>6</v>
+          <t>Wohnfläche (m²)</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>725</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>3 im 1. OG, 3 im Staffelgeschoss</t>
+          <t>8 Wohnungen: 5 × 83 m² im 1. OG, 3 × 103 m² im Staffelgeschoss</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Kaltmiete je Wohnung (€)</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="n">
-        <v>950</v>
+          <t>Kaltmiete je m² Wohnfläche (€)</t>
+        </is>
+      </c>
+      <c r="B26" s="11">
+        <f>950/85</f>
+        <v/>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Annahme des Bauherrn, Markt ca. 11 €/m²</t>
+          <t>950 € für 85 m² (Annahme des Bauherrn), Markt ca. 11 €/m²</t>
         </is>
       </c>
     </row>
@@ -924,11 +926,11 @@
         </is>
       </c>
       <c r="B35" s="6" t="n">
-        <v>280</v>
+        <v>460</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Zimmerei, Terrasse rundum</t>
+          <t>Zimmerei, schmale Terrasse (0,8 m) rundum</t>
         </is>
       </c>
     </row>
@@ -954,7 +956,7 @@
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
@@ -989,6 +991,45 @@
       <c r="C39" s="2" t="inlineStr">
         <is>
           <t>Bekanntenpreis, noch offen (z. B. 5 % oder 10 %)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Büro im EG</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="n"/>
+      <c r="C41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Büro-Fläche (m²)</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>vermietet</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Büro-Miete je m² (€)</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Annahme</t>
         </is>
       </c>
     </row>
@@ -1019,17 +1060,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Posten</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Betrag</t>
         </is>
       </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>Rechnung</t>
         </is>
@@ -1041,7 +1082,7 @@
           <t>Grundstück</t>
         </is>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="14">
         <f>Annahmen!B4*Annahmen!B5</f>
         <v/>
       </c>
@@ -1057,7 +1098,7 @@
           <t>Grunderwerbsteuer</t>
         </is>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="14">
         <f>B4*Annahmen!B6</f>
         <v/>
       </c>
@@ -1069,7 +1110,7 @@
           <t>Notar und Grundbuch</t>
         </is>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="14">
         <f>B4*Annahmen!B7</f>
         <v/>
       </c>
@@ -1081,7 +1122,7 @@
           <t>Grundstück gesamt</t>
         </is>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="14">
         <f>SUM(B4:B6)</f>
         <v/>
       </c>
@@ -1093,7 +1134,7 @@
           <t>Bau</t>
         </is>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="14">
         <f>(Annahmen!B8*Annahmen!B9-Annahmen!B35*Annahmen!B36+Annahmen!B37*Annahmen!B38)*(1-Annahmen!B39)</f>
         <v/>
       </c>
@@ -1109,7 +1150,7 @@
           <t>Baunebenkosten</t>
         </is>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="14">
         <f>B8*Annahmen!B10</f>
         <v/>
       </c>
@@ -1121,7 +1162,7 @@
           <t>Bau gesamt</t>
         </is>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="14">
         <f>B8+B9</f>
         <v/>
       </c>
@@ -1133,19 +1174,19 @@
           <t>Gastro-Ausbau</t>
         </is>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="14">
         <f>Annahmen!B11</f>
         <v/>
       </c>
       <c r="C11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="16">
         <f>B7+B10+B11</f>
         <v/>
       </c>
@@ -1157,19 +1198,19 @@
           <t>Förderung (Zuschuss)</t>
         </is>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="14">
         <f>-B12*Annahmen!B12</f>
         <v/>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Kosten nach Förderung</t>
         </is>
       </c>
-      <c r="B14" s="15">
+      <c r="B14" s="16">
         <f>B12+B13</f>
         <v/>
       </c>
@@ -1181,7 +1222,7 @@
           <t>Kosten je m² BGF</t>
         </is>
       </c>
-      <c r="B15" s="13">
+      <c r="B15" s="14">
         <f>B14/Annahmen!B8</f>
         <v/>
       </c>
@@ -1193,7 +1234,7 @@
           <t>Grundstück nach Förderung (für den Kredit)</t>
         </is>
       </c>
-      <c r="B17" s="13">
+      <c r="B17" s="14">
         <f>B7*(1-Annahmen!B12)</f>
         <v/>
       </c>
@@ -1205,7 +1246,7 @@
           <t>Bau und Gastro nach Förderung (für den Kredit)</t>
         </is>
       </c>
-      <c r="B18" s="13">
+      <c r="B18" s="14">
         <f>(B10+B11)*(1-Annahmen!B12)</f>
         <v/>
       </c>
@@ -1251,37 +1292,37 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Monat</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Auszahlung</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>Zinsen</t>
         </is>
       </c>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>Bereitstellung</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
+      <c r="E4" s="13" t="inlineStr">
         <is>
           <t>Noch nicht abgerufen</t>
         </is>
       </c>
-      <c r="F4" s="12" t="inlineStr">
+      <c r="F4" s="13" t="inlineStr">
         <is>
           <t>Kredit am Monatsende</t>
         </is>
       </c>
-      <c r="H4" s="14" t="inlineStr">
+      <c r="H4" s="15" t="inlineStr">
         <is>
           <t>Ergebnis</t>
         </is>
@@ -1291,21 +1332,21 @@
       <c r="A5" t="n">
         <v>0</v>
       </c>
-      <c r="B5" s="16">
+      <c r="B5" s="17">
         <f>Kosten!B17</f>
         <v/>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="16" t="n">
+      <c r="D5" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="16">
+      <c r="E5" s="17">
         <f>Kosten!B18</f>
         <v/>
       </c>
-      <c r="F5" s="16">
+      <c r="F5" s="17">
         <f>B5</f>
         <v/>
       </c>
@@ -1314,7 +1355,7 @@
           <t>Zinsen in der Bauzeit</t>
         </is>
       </c>
-      <c r="I5" s="13">
+      <c r="I5" s="14">
         <f>SUM(C6:C20)</f>
         <v/>
       </c>
@@ -1323,23 +1364,23 @@
       <c r="A6" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="16">
+      <c r="B6" s="17">
         <f>Kosten!$B$18/Annahmen!$B$19</f>
         <v/>
       </c>
-      <c r="C6" s="16">
+      <c r="C6" s="17">
         <f>F5*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="17">
         <f>IF(A6&gt;=Annahmen!$B$21,E6*Annahmen!$B$20/12,0)</f>
         <v/>
       </c>
-      <c r="E6" s="16">
+      <c r="E6" s="17">
         <f>Kosten!B18</f>
         <v/>
       </c>
-      <c r="F6" s="16">
+      <c r="F6" s="17">
         <f>F5+C6+D6+B6</f>
         <v/>
       </c>
@@ -1348,7 +1389,7 @@
           <t>Bereitstellungszinsen</t>
         </is>
       </c>
-      <c r="I6" s="13">
+      <c r="I6" s="14">
         <f>SUM(D6:D20)</f>
         <v/>
       </c>
@@ -1357,23 +1398,23 @@
       <c r="A7" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="17">
         <f>Kosten!$B$18/Annahmen!$B$19</f>
         <v/>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="17">
         <f>F6*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="17">
         <f>IF(A7&gt;=Annahmen!$B$21,E7*Annahmen!$B$20/12,0)</f>
         <v/>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="17">
         <f>E6-B6</f>
         <v/>
       </c>
-      <c r="F7" s="16">
+      <c r="F7" s="17">
         <f>F6+C7+D7+B7</f>
         <v/>
       </c>
@@ -1382,7 +1423,7 @@
           <t>Zinsen im Aufschub-Jahr</t>
         </is>
       </c>
-      <c r="I7" s="13">
+      <c r="I7" s="14">
         <f>SUM(C24:C35)</f>
         <v/>
       </c>
@@ -1391,32 +1432,32 @@
       <c r="A8" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="17">
         <f>Kosten!$B$18/Annahmen!$B$19</f>
         <v/>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="17">
         <f>F7*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="17">
         <f>IF(A8&gt;=Annahmen!$B$21,E8*Annahmen!$B$20/12,0)</f>
         <v/>
       </c>
-      <c r="E8" s="16">
+      <c r="E8" s="17">
         <f>E7-B7</f>
         <v/>
       </c>
-      <c r="F8" s="16">
+      <c r="F8" s="17">
         <f>F7+C8+D8+B8</f>
         <v/>
       </c>
-      <c r="H8" s="14" t="inlineStr">
+      <c r="H8" s="15" t="inlineStr">
         <is>
           <t>Kredit bei Start der Rate</t>
         </is>
       </c>
-      <c r="I8" s="15">
+      <c r="I8" s="16">
         <f>F35</f>
         <v/>
       </c>
@@ -1425,32 +1466,32 @@
       <c r="A9" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="17">
         <f>Kosten!$B$18/Annahmen!$B$19</f>
         <v/>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="17">
         <f>F8*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="17">
         <f>IF(A9&gt;=Annahmen!$B$21,E9*Annahmen!$B$20/12,0)</f>
         <v/>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="17">
         <f>E8-B8</f>
         <v/>
       </c>
-      <c r="F9" s="16">
+      <c r="F9" s="17">
         <f>F8+C9+D9+B9</f>
         <v/>
       </c>
-      <c r="H9" s="14" t="inlineStr">
+      <c r="H9" s="15" t="inlineStr">
         <is>
           <t>Rate pro Monat</t>
         </is>
       </c>
-      <c r="I9" s="15">
+      <c r="I9" s="16">
         <f>F35*(Annahmen!B17+Annahmen!B18)/12</f>
         <v/>
       </c>
@@ -1459,23 +1500,23 @@
       <c r="A10" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="17">
         <f>Kosten!$B$18/Annahmen!$B$19</f>
         <v/>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="17">
         <f>F9*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="17">
         <f>IF(A10&gt;=Annahmen!$B$21,E10*Annahmen!$B$20/12,0)</f>
         <v/>
       </c>
-      <c r="E10" s="16">
+      <c r="E10" s="17">
         <f>E9-B9</f>
         <v/>
       </c>
-      <c r="F10" s="16">
+      <c r="F10" s="17">
         <f>F9+C10+D10+B10</f>
         <v/>
       </c>
@@ -1484,7 +1525,7 @@
           <t xml:space="preserve">   davon Zinsen</t>
         </is>
       </c>
-      <c r="I10" s="13">
+      <c r="I10" s="14">
         <f>F35*Annahmen!B17/12</f>
         <v/>
       </c>
@@ -1493,23 +1534,23 @@
       <c r="A11" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="17">
         <f>Kosten!$B$18/Annahmen!$B$19</f>
         <v/>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="17">
         <f>F10*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="17">
         <f>IF(A11&gt;=Annahmen!$B$21,E11*Annahmen!$B$20/12,0)</f>
         <v/>
       </c>
-      <c r="E11" s="16">
+      <c r="E11" s="17">
         <f>E10-B10</f>
         <v/>
       </c>
-      <c r="F11" s="16">
+      <c r="F11" s="17">
         <f>F10+C11+D11+B11</f>
         <v/>
       </c>
@@ -1518,7 +1559,7 @@
           <t xml:space="preserve">   davon Tilgung</t>
         </is>
       </c>
-      <c r="I11" s="13">
+      <c r="I11" s="14">
         <f>F35*Annahmen!B18/12</f>
         <v/>
       </c>
@@ -1527,23 +1568,23 @@
       <c r="A12" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="17">
         <f>Kosten!$B$18/Annahmen!$B$19</f>
         <v/>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="17">
         <f>F11*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="17">
         <f>IF(A12&gt;=Annahmen!$B$21,E12*Annahmen!$B$20/12,0)</f>
         <v/>
       </c>
-      <c r="E12" s="16">
+      <c r="E12" s="17">
         <f>E11-B11</f>
         <v/>
       </c>
-      <c r="F12" s="16">
+      <c r="F12" s="17">
         <f>F11+C12+D12+B12</f>
         <v/>
       </c>
@@ -1552,23 +1593,23 @@
       <c r="A13" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="16">
+      <c r="B13" s="17">
         <f>Kosten!$B$18/Annahmen!$B$19</f>
         <v/>
       </c>
-      <c r="C13" s="16">
+      <c r="C13" s="17">
         <f>F12*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D13" s="16">
+      <c r="D13" s="17">
         <f>IF(A13&gt;=Annahmen!$B$21,E13*Annahmen!$B$20/12,0)</f>
         <v/>
       </c>
-      <c r="E13" s="16">
+      <c r="E13" s="17">
         <f>E12-B12</f>
         <v/>
       </c>
-      <c r="F13" s="16">
+      <c r="F13" s="17">
         <f>F12+C13+D13+B13</f>
         <v/>
       </c>
@@ -1577,23 +1618,23 @@
       <c r="A14" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="17">
         <f>Kosten!$B$18/Annahmen!$B$19</f>
         <v/>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="17">
         <f>F13*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D14" s="16">
+      <c r="D14" s="17">
         <f>IF(A14&gt;=Annahmen!$B$21,E14*Annahmen!$B$20/12,0)</f>
         <v/>
       </c>
-      <c r="E14" s="16">
+      <c r="E14" s="17">
         <f>E13-B13</f>
         <v/>
       </c>
-      <c r="F14" s="16">
+      <c r="F14" s="17">
         <f>F13+C14+D14+B14</f>
         <v/>
       </c>
@@ -1602,23 +1643,23 @@
       <c r="A15" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="16">
+      <c r="B15" s="17">
         <f>Kosten!$B$18/Annahmen!$B$19</f>
         <v/>
       </c>
-      <c r="C15" s="16">
+      <c r="C15" s="17">
         <f>F14*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="17">
         <f>IF(A15&gt;=Annahmen!$B$21,E15*Annahmen!$B$20/12,0)</f>
         <v/>
       </c>
-      <c r="E15" s="16">
+      <c r="E15" s="17">
         <f>E14-B14</f>
         <v/>
       </c>
-      <c r="F15" s="16">
+      <c r="F15" s="17">
         <f>F14+C15+D15+B15</f>
         <v/>
       </c>
@@ -1627,23 +1668,23 @@
       <c r="A16" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="17">
         <f>Kosten!$B$18/Annahmen!$B$19</f>
         <v/>
       </c>
-      <c r="C16" s="16">
+      <c r="C16" s="17">
         <f>F15*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="17">
         <f>IF(A16&gt;=Annahmen!$B$21,E16*Annahmen!$B$20/12,0)</f>
         <v/>
       </c>
-      <c r="E16" s="16">
+      <c r="E16" s="17">
         <f>E15-B15</f>
         <v/>
       </c>
-      <c r="F16" s="16">
+      <c r="F16" s="17">
         <f>F15+C16+D16+B16</f>
         <v/>
       </c>
@@ -1652,23 +1693,23 @@
       <c r="A17" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="16">
+      <c r="B17" s="17">
         <f>Kosten!$B$18/Annahmen!$B$19</f>
         <v/>
       </c>
-      <c r="C17" s="16">
+      <c r="C17" s="17">
         <f>F16*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D17" s="16">
+      <c r="D17" s="17">
         <f>IF(A17&gt;=Annahmen!$B$21,E17*Annahmen!$B$20/12,0)</f>
         <v/>
       </c>
-      <c r="E17" s="16">
+      <c r="E17" s="17">
         <f>E16-B16</f>
         <v/>
       </c>
-      <c r="F17" s="16">
+      <c r="F17" s="17">
         <f>F16+C17+D17+B17</f>
         <v/>
       </c>
@@ -1677,23 +1718,23 @@
       <c r="A18" t="n">
         <v>13</v>
       </c>
-      <c r="B18" s="16">
+      <c r="B18" s="17">
         <f>Kosten!$B$18/Annahmen!$B$19</f>
         <v/>
       </c>
-      <c r="C18" s="16">
+      <c r="C18" s="17">
         <f>F17*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D18" s="16">
+      <c r="D18" s="17">
         <f>IF(A18&gt;=Annahmen!$B$21,E18*Annahmen!$B$20/12,0)</f>
         <v/>
       </c>
-      <c r="E18" s="16">
+      <c r="E18" s="17">
         <f>E17-B17</f>
         <v/>
       </c>
-      <c r="F18" s="16">
+      <c r="F18" s="17">
         <f>F17+C18+D18+B18</f>
         <v/>
       </c>
@@ -1702,23 +1743,23 @@
       <c r="A19" t="n">
         <v>14</v>
       </c>
-      <c r="B19" s="16">
+      <c r="B19" s="17">
         <f>Kosten!$B$18/Annahmen!$B$19</f>
         <v/>
       </c>
-      <c r="C19" s="16">
+      <c r="C19" s="17">
         <f>F18*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D19" s="16">
+      <c r="D19" s="17">
         <f>IF(A19&gt;=Annahmen!$B$21,E19*Annahmen!$B$20/12,0)</f>
         <v/>
       </c>
-      <c r="E19" s="16">
+      <c r="E19" s="17">
         <f>E18-B18</f>
         <v/>
       </c>
-      <c r="F19" s="16">
+      <c r="F19" s="17">
         <f>F18+C19+D19+B19</f>
         <v/>
       </c>
@@ -1727,61 +1768,61 @@
       <c r="A20" t="n">
         <v>15</v>
       </c>
-      <c r="B20" s="16">
+      <c r="B20" s="17">
         <f>Kosten!$B$18/Annahmen!$B$19</f>
         <v/>
       </c>
-      <c r="C20" s="16">
+      <c r="C20" s="17">
         <f>F19*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D20" s="16">
+      <c r="D20" s="17">
         <f>IF(A20&gt;=Annahmen!$B$21,E20*Annahmen!$B$20/12,0)</f>
         <v/>
       </c>
-      <c r="E20" s="16">
+      <c r="E20" s="17">
         <f>E19-B19</f>
         <v/>
       </c>
-      <c r="F20" s="16">
+      <c r="F20" s="17">
         <f>F19+C20+D20+B20</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="16" t="n"/>
-      <c r="C21" s="16" t="n"/>
-      <c r="D21" s="16" t="n"/>
-      <c r="E21" s="16" t="n"/>
-      <c r="F21" s="16" t="n"/>
+      <c r="B21" s="17" t="n"/>
+      <c r="C21" s="17" t="n"/>
+      <c r="D21" s="17" t="n"/>
+      <c r="E21" s="17" t="n"/>
+      <c r="F21" s="17" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>Raten-Aufschub: nur Zinsen laufen auf</t>
         </is>
       </c>
-      <c r="B22" s="16" t="n"/>
-      <c r="C22" s="16" t="n"/>
-      <c r="D22" s="16" t="n"/>
-      <c r="E22" s="16" t="n"/>
-      <c r="F22" s="16" t="n"/>
+      <c r="B22" s="17" t="n"/>
+      <c r="C22" s="17" t="n"/>
+      <c r="D22" s="17" t="n"/>
+      <c r="E22" s="17" t="n"/>
+      <c r="F22" s="17" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>Monat</t>
         </is>
       </c>
-      <c r="B23" s="17" t="inlineStr"/>
-      <c r="C23" s="17" t="inlineStr">
+      <c r="B23" s="18" t="inlineStr"/>
+      <c r="C23" s="18" t="inlineStr">
         <is>
           <t>Zinsen</t>
         </is>
       </c>
-      <c r="D23" s="17" t="inlineStr"/>
-      <c r="E23" s="17" t="inlineStr"/>
-      <c r="F23" s="17" t="inlineStr">
+      <c r="D23" s="18" t="inlineStr"/>
+      <c r="E23" s="18" t="inlineStr"/>
+      <c r="F23" s="18" t="inlineStr">
         <is>
           <t>Kredit am Monatsende</t>
         </is>
@@ -1791,14 +1832,14 @@
       <c r="A24" t="n">
         <v>1</v>
       </c>
-      <c r="B24" s="16" t="n"/>
-      <c r="C24" s="16">
+      <c r="B24" s="17" t="n"/>
+      <c r="C24" s="17">
         <f>F20*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D24" s="16" t="n"/>
-      <c r="E24" s="16" t="n"/>
-      <c r="F24" s="16">
+      <c r="D24" s="17" t="n"/>
+      <c r="E24" s="17" t="n"/>
+      <c r="F24" s="17">
         <f>F20+C24</f>
         <v/>
       </c>
@@ -1807,14 +1848,14 @@
       <c r="A25" t="n">
         <v>2</v>
       </c>
-      <c r="B25" s="16" t="n"/>
-      <c r="C25" s="16">
+      <c r="B25" s="17" t="n"/>
+      <c r="C25" s="17">
         <f>F24*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D25" s="16" t="n"/>
-      <c r="E25" s="16" t="n"/>
-      <c r="F25" s="16">
+      <c r="D25" s="17" t="n"/>
+      <c r="E25" s="17" t="n"/>
+      <c r="F25" s="17">
         <f>F24+C25</f>
         <v/>
       </c>
@@ -1823,14 +1864,14 @@
       <c r="A26" t="n">
         <v>3</v>
       </c>
-      <c r="B26" s="16" t="n"/>
-      <c r="C26" s="16">
+      <c r="B26" s="17" t="n"/>
+      <c r="C26" s="17">
         <f>F25*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D26" s="16" t="n"/>
-      <c r="E26" s="16" t="n"/>
-      <c r="F26" s="16">
+      <c r="D26" s="17" t="n"/>
+      <c r="E26" s="17" t="n"/>
+      <c r="F26" s="17">
         <f>F25+C26</f>
         <v/>
       </c>
@@ -1839,14 +1880,14 @@
       <c r="A27" t="n">
         <v>4</v>
       </c>
-      <c r="B27" s="16" t="n"/>
-      <c r="C27" s="16">
+      <c r="B27" s="17" t="n"/>
+      <c r="C27" s="17">
         <f>F26*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D27" s="16" t="n"/>
-      <c r="E27" s="16" t="n"/>
-      <c r="F27" s="16">
+      <c r="D27" s="17" t="n"/>
+      <c r="E27" s="17" t="n"/>
+      <c r="F27" s="17">
         <f>F26+C27</f>
         <v/>
       </c>
@@ -1855,14 +1896,14 @@
       <c r="A28" t="n">
         <v>5</v>
       </c>
-      <c r="B28" s="16" t="n"/>
-      <c r="C28" s="16">
+      <c r="B28" s="17" t="n"/>
+      <c r="C28" s="17">
         <f>F27*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D28" s="16" t="n"/>
-      <c r="E28" s="16" t="n"/>
-      <c r="F28" s="16">
+      <c r="D28" s="17" t="n"/>
+      <c r="E28" s="17" t="n"/>
+      <c r="F28" s="17">
         <f>F27+C28</f>
         <v/>
       </c>
@@ -1871,14 +1912,14 @@
       <c r="A29" t="n">
         <v>6</v>
       </c>
-      <c r="B29" s="16" t="n"/>
-      <c r="C29" s="16">
+      <c r="B29" s="17" t="n"/>
+      <c r="C29" s="17">
         <f>F28*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D29" s="16" t="n"/>
-      <c r="E29" s="16" t="n"/>
-      <c r="F29" s="16">
+      <c r="D29" s="17" t="n"/>
+      <c r="E29" s="17" t="n"/>
+      <c r="F29" s="17">
         <f>F28+C29</f>
         <v/>
       </c>
@@ -1887,14 +1928,14 @@
       <c r="A30" t="n">
         <v>7</v>
       </c>
-      <c r="B30" s="16" t="n"/>
-      <c r="C30" s="16">
+      <c r="B30" s="17" t="n"/>
+      <c r="C30" s="17">
         <f>F29*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D30" s="16" t="n"/>
-      <c r="E30" s="16" t="n"/>
-      <c r="F30" s="16">
+      <c r="D30" s="17" t="n"/>
+      <c r="E30" s="17" t="n"/>
+      <c r="F30" s="17">
         <f>F29+C30</f>
         <v/>
       </c>
@@ -1903,14 +1944,14 @@
       <c r="A31" t="n">
         <v>8</v>
       </c>
-      <c r="B31" s="16" t="n"/>
-      <c r="C31" s="16">
+      <c r="B31" s="17" t="n"/>
+      <c r="C31" s="17">
         <f>F30*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D31" s="16" t="n"/>
-      <c r="E31" s="16" t="n"/>
-      <c r="F31" s="16">
+      <c r="D31" s="17" t="n"/>
+      <c r="E31" s="17" t="n"/>
+      <c r="F31" s="17">
         <f>F30+C31</f>
         <v/>
       </c>
@@ -1919,14 +1960,14 @@
       <c r="A32" t="n">
         <v>9</v>
       </c>
-      <c r="B32" s="16" t="n"/>
-      <c r="C32" s="16">
+      <c r="B32" s="17" t="n"/>
+      <c r="C32" s="17">
         <f>F31*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D32" s="16" t="n"/>
-      <c r="E32" s="16" t="n"/>
-      <c r="F32" s="16">
+      <c r="D32" s="17" t="n"/>
+      <c r="E32" s="17" t="n"/>
+      <c r="F32" s="17">
         <f>F31+C32</f>
         <v/>
       </c>
@@ -1935,14 +1976,14 @@
       <c r="A33" t="n">
         <v>10</v>
       </c>
-      <c r="B33" s="16" t="n"/>
-      <c r="C33" s="16">
+      <c r="B33" s="17" t="n"/>
+      <c r="C33" s="17">
         <f>F32*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D33" s="16" t="n"/>
-      <c r="E33" s="16" t="n"/>
-      <c r="F33" s="16">
+      <c r="D33" s="17" t="n"/>
+      <c r="E33" s="17" t="n"/>
+      <c r="F33" s="17">
         <f>F32+C33</f>
         <v/>
       </c>
@@ -1951,14 +1992,14 @@
       <c r="A34" t="n">
         <v>11</v>
       </c>
-      <c r="B34" s="16" t="n"/>
-      <c r="C34" s="16">
+      <c r="B34" s="17" t="n"/>
+      <c r="C34" s="17">
         <f>F33*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D34" s="16" t="n"/>
-      <c r="E34" s="16" t="n"/>
-      <c r="F34" s="16">
+      <c r="D34" s="17" t="n"/>
+      <c r="E34" s="17" t="n"/>
+      <c r="F34" s="17">
         <f>F33+C34</f>
         <v/>
       </c>
@@ -1967,14 +2008,14 @@
       <c r="A35" t="n">
         <v>12</v>
       </c>
-      <c r="B35" s="16" t="n"/>
-      <c r="C35" s="16">
+      <c r="B35" s="17" t="n"/>
+      <c r="C35" s="17">
         <f>F34*Annahmen!$B$17/12</f>
         <v/>
       </c>
-      <c r="D35" s="16" t="n"/>
-      <c r="E35" s="16" t="n"/>
-      <c r="F35" s="16">
+      <c r="D35" s="17" t="n"/>
+      <c r="E35" s="17" t="n"/>
+      <c r="F35" s="17">
         <f>F34+C35</f>
         <v/>
       </c>
@@ -2012,12 +2053,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Posten</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>pro Monat</t>
         </is>
@@ -2026,11 +2067,11 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Wohnungen (Kaltmiete)</t>
-        </is>
-      </c>
-      <c r="B5" s="13">
-        <f>Annahmen!B25*Annahmen!B26</f>
+          <t>Wohnungen und Büro (Kaltmiete)</t>
+        </is>
+      </c>
+      <c r="B5" s="14">
+        <f>Annahmen!B25*Annahmen!B26+Annahmen!B42*Annahmen!B43</f>
         <v/>
       </c>
     </row>
@@ -2040,7 +2081,7 @@
           <t>Gastro-Pacht</t>
         </is>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="14">
         <f>Annahmen!B27*Annahmen!B28</f>
         <v/>
       </c>
@@ -2051,7 +2092,7 @@
           <t>Miete und Pacht gesamt</t>
         </is>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="14">
         <f>B5+B6</f>
         <v/>
       </c>
@@ -2062,7 +2103,7 @@
           <t>Gastro-Gewinn nach Pacht</t>
         </is>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="14">
         <f>Annahmen!B30*Annahmen!B31-B6</f>
         <v/>
       </c>
@@ -2073,7 +2114,7 @@
           <t>Rate (Zinsen und Tilgung)</t>
         </is>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="14">
         <f>-Kredit!I9</f>
         <v/>
       </c>
@@ -2084,7 +2125,7 @@
           <t>Dein Lohn</t>
         </is>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="14">
         <f>-Annahmen!B32</f>
         <v/>
       </c>
@@ -2095,18 +2136,18 @@
           <t>Rücklagen</t>
         </is>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="14">
         <f>-B7*Annahmen!B29</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Ergebnis pro Monat</t>
         </is>
       </c>
-      <c r="B12" s="18">
+      <c r="B12" s="19">
         <f>B5+B6+B8+B9+B10+B11</f>
         <v/>
       </c>
@@ -2117,18 +2158,18 @@
           <t>Ergebnis pro Jahr</t>
         </is>
       </c>
-      <c r="B13" s="19">
+      <c r="B13" s="20">
         <f>B12*12</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Break-even Gastro-Umsatz (Ergebnis = 0, abzüglich Lohn aus Annahmen)</t>
         </is>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="16">
         <f>(Annahmen!B32+Kredit!I9+B7*Annahmen!B29-B7+B6)/Annahmen!B31</f>
         <v/>
       </c>
@@ -2179,320 +2220,320 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Förderung</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>Rate Plan 3,3 %</t>
         </is>
       </c>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>Ergebnis Plan</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
+      <c r="E4" s="13" t="inlineStr">
         <is>
           <t>Rate Ausgang 4,0 %</t>
         </is>
       </c>
-      <c r="F4" s="12" t="inlineStr">
+      <c r="F4" s="13" t="inlineStr">
         <is>
           <t>Ergebnis Ausgang</t>
         </is>
       </c>
-      <c r="G4" s="12" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>Break-even Umsatz Plan</t>
         </is>
       </c>
-      <c r="H4" s="12" t="inlineStr">
+      <c r="H4" s="13" t="inlineStr">
         <is>
           <t>Break-even Umsatz Ausgang</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="n">
+      <c r="A5" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="B5" s="16" t="n">
-        <v>2716271</v>
-      </c>
-      <c r="C5" s="16" t="n">
-        <v>10345.03</v>
-      </c>
-      <c r="D5" s="21" t="n">
-        <v>9686.969999999999</v>
-      </c>
-      <c r="E5" s="16" t="n">
-        <v>12168.04</v>
-      </c>
-      <c r="F5" s="21" t="n">
-        <v>7863.96</v>
-      </c>
-      <c r="G5" s="16" t="n">
-        <v>18239.43</v>
-      </c>
-      <c r="H5" s="16" t="n">
-        <v>24216.52</v>
+      <c r="B5" s="17" t="n">
+        <v>4108116</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>15639.22</v>
+      </c>
+      <c r="D5" s="22" t="n">
+        <v>7905.43</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>18392.63</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>5152.01</v>
+      </c>
+      <c r="G5" s="17" t="n">
+        <v>24080.56</v>
+      </c>
+      <c r="H5" s="17" t="n">
+        <v>33108.15</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="n">
+      <c r="A6" s="21" t="n">
         <v>0.05</v>
       </c>
-      <c r="B6" s="16" t="n">
-        <v>2580457.45</v>
-      </c>
-      <c r="C6" s="16" t="n">
-        <v>9827.780000000001</v>
-      </c>
-      <c r="D6" s="21" t="n">
-        <v>10204.22</v>
-      </c>
-      <c r="E6" s="16" t="n">
-        <v>11559.64</v>
-      </c>
-      <c r="F6" s="21" t="n">
-        <v>8472.360000000001</v>
-      </c>
-      <c r="G6" s="16" t="n">
-        <v>16543.53</v>
-      </c>
-      <c r="H6" s="16" t="n">
-        <v>22221.76</v>
+      <c r="B6" s="17" t="n">
+        <v>3902710.2</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>14857.26</v>
+      </c>
+      <c r="D6" s="22" t="n">
+        <v>8687.389999999999</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>17473</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>6071.65</v>
+      </c>
+      <c r="G6" s="17" t="n">
+        <v>21516.75</v>
+      </c>
+      <c r="H6" s="17" t="n">
+        <v>30092.97</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="n">
+      <c r="A7" s="21" t="n">
         <v>0.1</v>
       </c>
-      <c r="B7" s="16" t="n">
-        <v>2444643.9</v>
-      </c>
-      <c r="C7" s="16" t="n">
-        <v>9310.52</v>
-      </c>
-      <c r="D7" s="21" t="n">
-        <v>10721.48</v>
-      </c>
-      <c r="E7" s="16" t="n">
-        <v>10951.24</v>
-      </c>
-      <c r="F7" s="21" t="n">
-        <v>9080.76</v>
-      </c>
-      <c r="G7" s="16" t="n">
-        <v>14847.62</v>
-      </c>
-      <c r="H7" s="16" t="n">
-        <v>20227</v>
+      <c r="B7" s="17" t="n">
+        <v>3697304.4</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>14075.3</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>9469.35</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>16553.37</v>
+      </c>
+      <c r="F7" s="22" t="n">
+        <v>6991.28</v>
+      </c>
+      <c r="G7" s="17" t="n">
+        <v>18952.95</v>
+      </c>
+      <c r="H7" s="17" t="n">
+        <v>27077.78</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="n">
+      <c r="A8" s="21" t="n">
         <v>0.15</v>
       </c>
-      <c r="B8" s="16" t="n">
-        <v>2308830.35</v>
-      </c>
-      <c r="C8" s="16" t="n">
-        <v>8793.27</v>
-      </c>
-      <c r="D8" s="21" t="n">
-        <v>11238.73</v>
-      </c>
-      <c r="E8" s="16" t="n">
-        <v>10342.83</v>
-      </c>
-      <c r="F8" s="21" t="n">
-        <v>9689.17</v>
-      </c>
-      <c r="G8" s="16" t="n">
-        <v>13151.72</v>
-      </c>
-      <c r="H8" s="16" t="n">
-        <v>18232.24</v>
+      <c r="B8" s="17" t="n">
+        <v>3491898.6</v>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>13293.33</v>
+      </c>
+      <c r="D8" s="22" t="n">
+        <v>10251.31</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>15633.74</v>
+      </c>
+      <c r="F8" s="22" t="n">
+        <v>7910.91</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <v>16389.14</v>
+      </c>
+      <c r="H8" s="17" t="n">
+        <v>24062.6</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="n">
+      <c r="A9" s="21" t="n">
         <v>0.2</v>
       </c>
-      <c r="B9" s="16" t="n">
-        <v>2173016.8</v>
-      </c>
-      <c r="C9" s="16" t="n">
-        <v>8276.02</v>
-      </c>
-      <c r="D9" s="21" t="n">
-        <v>11755.98</v>
-      </c>
-      <c r="E9" s="16" t="n">
-        <v>9734.43</v>
-      </c>
-      <c r="F9" s="21" t="n">
-        <v>10297.57</v>
-      </c>
-      <c r="G9" s="16" t="n">
-        <v>11455.81</v>
-      </c>
-      <c r="H9" s="16" t="n">
-        <v>16237.48</v>
+      <c r="B9" s="17" t="n">
+        <v>3286492.8</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>12511.37</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>11033.27</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>14714.11</v>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>8830.540000000001</v>
+      </c>
+      <c r="G9" s="17" t="n">
+        <v>13825.33</v>
+      </c>
+      <c r="H9" s="17" t="n">
+        <v>21047.41</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="n">
+      <c r="A10" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="B10" s="16" t="n">
-        <v>2037203.25</v>
-      </c>
-      <c r="C10" s="16" t="n">
-        <v>7758.77</v>
-      </c>
-      <c r="D10" s="21" t="n">
-        <v>12273.23</v>
-      </c>
-      <c r="E10" s="16" t="n">
-        <v>9126.030000000001</v>
-      </c>
-      <c r="F10" s="21" t="n">
-        <v>10905.97</v>
-      </c>
-      <c r="G10" s="16" t="n">
-        <v>9759.9</v>
-      </c>
-      <c r="H10" s="16" t="n">
-        <v>14242.72</v>
+      <c r="B10" s="17" t="n">
+        <v>3081087</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>11729.41</v>
+      </c>
+      <c r="D10" s="22" t="n">
+        <v>11815.23</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>13794.48</v>
+      </c>
+      <c r="F10" s="22" t="n">
+        <v>9750.17</v>
+      </c>
+      <c r="G10" s="17" t="n">
+        <v>11261.53</v>
+      </c>
+      <c r="H10" s="17" t="n">
+        <v>18032.22</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Ergebnis pro Monat (ohne Lohn des Bauherrn), Plan 3,3 %, je Gastro-Umsatz</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Förderung</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>40.000 €</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>45.000 €</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>50.000 €</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="E13" s="13" t="inlineStr">
         <is>
           <t>55.000 €</t>
         </is>
       </c>
-      <c r="F13" s="12" t="inlineStr">
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>60.000 €</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="n">
+      <c r="A14" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="B14" s="21" t="n">
-        <v>6636.97</v>
-      </c>
-      <c r="C14" s="21" t="n">
-        <v>8161.97</v>
-      </c>
-      <c r="D14" s="21" t="n">
-        <v>9686.969999999999</v>
-      </c>
-      <c r="E14" s="21" t="n">
-        <v>11211.97</v>
-      </c>
-      <c r="F14" s="21" t="n">
-        <v>12736.97</v>
+      <c r="B14" s="22" t="n">
+        <v>4855.43</v>
+      </c>
+      <c r="C14" s="22" t="n">
+        <v>6380.43</v>
+      </c>
+      <c r="D14" s="22" t="n">
+        <v>7905.43</v>
+      </c>
+      <c r="E14" s="22" t="n">
+        <v>9430.43</v>
+      </c>
+      <c r="F14" s="22" t="n">
+        <v>10955.43</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="n">
+      <c r="A15" s="21" t="n">
         <v>0.1</v>
       </c>
-      <c r="B15" s="21" t="n">
-        <v>7671.48</v>
-      </c>
-      <c r="C15" s="21" t="n">
-        <v>9196.48</v>
-      </c>
-      <c r="D15" s="21" t="n">
-        <v>10721.48</v>
-      </c>
-      <c r="E15" s="21" t="n">
-        <v>12246.48</v>
-      </c>
-      <c r="F15" s="21" t="n">
-        <v>13771.48</v>
+      <c r="B15" s="22" t="n">
+        <v>6419.35</v>
+      </c>
+      <c r="C15" s="22" t="n">
+        <v>7944.35</v>
+      </c>
+      <c r="D15" s="22" t="n">
+        <v>9469.35</v>
+      </c>
+      <c r="E15" s="22" t="n">
+        <v>10994.35</v>
+      </c>
+      <c r="F15" s="22" t="n">
+        <v>12519.35</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="n">
+      <c r="A16" s="21" t="n">
         <v>0.15</v>
       </c>
-      <c r="B16" s="21" t="n">
-        <v>8188.73</v>
-      </c>
-      <c r="C16" s="21" t="n">
-        <v>9713.73</v>
-      </c>
-      <c r="D16" s="21" t="n">
-        <v>11238.73</v>
-      </c>
-      <c r="E16" s="21" t="n">
-        <v>12763.73</v>
-      </c>
-      <c r="F16" s="21" t="n">
-        <v>14288.73</v>
+      <c r="B16" s="22" t="n">
+        <v>7201.31</v>
+      </c>
+      <c r="C16" s="22" t="n">
+        <v>8726.309999999999</v>
+      </c>
+      <c r="D16" s="22" t="n">
+        <v>10251.31</v>
+      </c>
+      <c r="E16" s="22" t="n">
+        <v>11776.31</v>
+      </c>
+      <c r="F16" s="22" t="n">
+        <v>13301.31</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="n">
+      <c r="A17" s="21" t="n">
         <v>0.2</v>
       </c>
-      <c r="B17" s="21" t="n">
-        <v>8705.98</v>
-      </c>
-      <c r="C17" s="21" t="n">
-        <v>10230.98</v>
-      </c>
-      <c r="D17" s="21" t="n">
-        <v>11755.98</v>
-      </c>
-      <c r="E17" s="21" t="n">
-        <v>13280.98</v>
-      </c>
-      <c r="F17" s="21" t="n">
-        <v>14805.98</v>
+      <c r="B17" s="22" t="n">
+        <v>7983.27</v>
+      </c>
+      <c r="C17" s="22" t="n">
+        <v>9508.27</v>
+      </c>
+      <c r="D17" s="22" t="n">
+        <v>11033.27</v>
+      </c>
+      <c r="E17" s="22" t="n">
+        <v>12558.27</v>
+      </c>
+      <c r="F17" s="22" t="n">
+        <v>14083.27</v>
       </c>
     </row>
   </sheetData>
@@ -2506,7 +2547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -2536,48 +2577,48 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr"/>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr"/>
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>A: 1. OG 85 m²</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>A: Staffel 63 m²</t>
         </is>
       </c>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>A: Gastro (Du)</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>B: 1. OG 85 m²</t>
-        </is>
-      </c>
-      <c r="F4" s="12" t="inlineStr">
-        <is>
-          <t>B: Staffel 63 m²</t>
-        </is>
-      </c>
-      <c r="G4" s="12" t="inlineStr">
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>B: 1. OG 83 m²</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>B: Staffel 103 m²</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>B: Gastro + Büro (Du)</t>
         </is>
       </c>
-      <c r="H4" s="12" t="inlineStr">
-        <is>
-          <t>C: Regelgeschoss 85 m²</t>
-        </is>
-      </c>
-      <c r="I4" s="12" t="inlineStr">
-        <is>
-          <t>C: Staffel 63 m²</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="inlineStr">
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>C: Regelgeschoss 83 m²</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>C: Staffel 103 m²</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr">
         <is>
           <t>C: Gastro + Büro (Du)</t>
         </is>
@@ -2589,31 +2630,31 @@
           <t>Preis (Selbstkosten)</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="17" t="n">
         <v>314624.67</v>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="17" t="n">
         <v>226174.33</v>
       </c>
-      <c r="D5" s="16" t="n">
+      <c r="D5" s="17" t="n">
         <v>1093874</v>
       </c>
-      <c r="E5" s="16" t="n">
-        <v>296791.94</v>
-      </c>
-      <c r="F5" s="16" t="n">
-        <v>216266.8</v>
-      </c>
-      <c r="G5" s="16" t="n">
+      <c r="E5" s="17" t="n">
+        <v>289808.6</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <v>353343.32</v>
+      </c>
+      <c r="G5" s="17" t="n">
         <v>1599043.01</v>
       </c>
-      <c r="H5" s="16" t="n">
-        <v>292386.83</v>
-      </c>
-      <c r="I5" s="16" t="n">
-        <v>212543.49</v>
-      </c>
-      <c r="J5" s="16" t="n">
+      <c r="H5" s="17" t="n">
+        <v>142753.57</v>
+      </c>
+      <c r="I5" s="17" t="n">
+        <v>347236.31</v>
+      </c>
+      <c r="J5" s="17" t="n">
         <v>1577535.69</v>
       </c>
     </row>
@@ -2623,32 +2664,32 @@
           <t>Rate pro Monat</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n">
-        <v>1198.26</v>
-      </c>
-      <c r="C6" s="16" t="n">
-        <v>861.39</v>
-      </c>
-      <c r="D6" s="16" t="n">
-        <v>4166.06</v>
-      </c>
-      <c r="E6" s="16" t="n">
-        <v>1130.34</v>
-      </c>
-      <c r="F6" s="16" t="n">
-        <v>823.66</v>
-      </c>
-      <c r="G6" s="16" t="n">
-        <v>6090.02</v>
-      </c>
-      <c r="H6" s="16" t="n">
-        <v>1113.57</v>
-      </c>
-      <c r="I6" s="16" t="n">
-        <v>809.48</v>
-      </c>
-      <c r="J6" s="16" t="n">
-        <v>6008.11</v>
+      <c r="B6" s="17" t="n">
+        <v>1197.75</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>861.02</v>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>4164.28</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>1103.27</v>
+      </c>
+      <c r="F6" s="17" t="n">
+        <v>1345.15</v>
+      </c>
+      <c r="G6" s="17" t="n">
+        <v>6087.41</v>
+      </c>
+      <c r="H6" s="17" t="n">
+        <v>543.45</v>
+      </c>
+      <c r="I6" s="17" t="n">
+        <v>1321.9</v>
+      </c>
+      <c r="J6" s="17" t="n">
+        <v>6005.53</v>
       </c>
     </row>
     <row r="7">
@@ -2657,31 +2698,31 @@
           <t>Einnahme nach Rücklagen / Gastro-Gewinn (+ Büro)</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="17" t="n">
         <v>855</v>
       </c>
-      <c r="C7" s="16" t="n">
-        <v>855</v>
-      </c>
-      <c r="D7" s="16" t="n">
+      <c r="C7" s="17" t="n">
+        <v>633.71</v>
+      </c>
+      <c r="D7" s="17" t="n">
         <v>15250</v>
       </c>
-      <c r="E7" s="16" t="n">
-        <v>855</v>
-      </c>
-      <c r="F7" s="16" t="n">
-        <v>855</v>
-      </c>
-      <c r="G7" s="16" t="n">
+      <c r="E7" s="17" t="n">
+        <v>834.88</v>
+      </c>
+      <c r="F7" s="17" t="n">
+        <v>1039.41</v>
+      </c>
+      <c r="G7" s="17" t="n">
         <v>16600</v>
       </c>
-      <c r="H7" s="16" t="n">
-        <v>855</v>
-      </c>
-      <c r="I7" s="16" t="n">
-        <v>855</v>
-      </c>
-      <c r="J7" s="16" t="n">
+      <c r="H7" s="17" t="n">
+        <v>417.44</v>
+      </c>
+      <c r="I7" s="17" t="n">
+        <v>1039.41</v>
+      </c>
+      <c r="J7" s="17" t="n">
         <v>16600</v>
       </c>
     </row>
@@ -2691,32 +2732,32 @@
           <t>Ergebnis pro Monat</t>
         </is>
       </c>
-      <c r="B8" s="21" t="n">
-        <v>-343.26</v>
-      </c>
-      <c r="C8" s="21" t="n">
-        <v>-6.39</v>
-      </c>
-      <c r="D8" s="21" t="n">
-        <v>11083.94</v>
-      </c>
-      <c r="E8" s="21" t="n">
-        <v>-275.34</v>
-      </c>
-      <c r="F8" s="21" t="n">
-        <v>31.34</v>
-      </c>
-      <c r="G8" s="21" t="n">
-        <v>10509.98</v>
-      </c>
-      <c r="H8" s="21" t="n">
-        <v>-258.57</v>
-      </c>
-      <c r="I8" s="21" t="n">
-        <v>45.52</v>
-      </c>
-      <c r="J8" s="21" t="n">
-        <v>10591.89</v>
+      <c r="B8" s="22" t="n">
+        <v>-342.75</v>
+      </c>
+      <c r="C8" s="22" t="n">
+        <v>-227.32</v>
+      </c>
+      <c r="D8" s="22" t="n">
+        <v>11085.72</v>
+      </c>
+      <c r="E8" s="22" t="n">
+        <v>-268.39</v>
+      </c>
+      <c r="F8" s="22" t="n">
+        <v>-305.73</v>
+      </c>
+      <c r="G8" s="22" t="n">
+        <v>10512.59</v>
+      </c>
+      <c r="H8" s="22" t="n">
+        <v>-126.01</v>
+      </c>
+      <c r="I8" s="22" t="n">
+        <v>-282.48</v>
+      </c>
+      <c r="J8" s="22" t="n">
+        <v>10594.47</v>
       </c>
     </row>
     <row r="9">
@@ -2725,23 +2766,23 @@
           <t>Preis für Ergebnis 0 €</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n">
-        <v>211220.58</v>
-      </c>
-      <c r="C9" s="16" t="n">
-        <v>211220.58</v>
-      </c>
-      <c r="E9" s="16" t="n">
-        <v>211220.58</v>
-      </c>
-      <c r="F9" s="16" t="n">
-        <v>211220.58</v>
-      </c>
-      <c r="H9" s="16" t="n">
-        <v>211220.58</v>
-      </c>
-      <c r="I9" s="16" t="n">
-        <v>211220.58</v>
+      <c r="B9" s="17" t="n">
+        <v>211401.81</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>156686.04</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>206427.65</v>
+      </c>
+      <c r="F9" s="17" t="n">
+        <v>256998.27</v>
+      </c>
+      <c r="H9" s="17" t="n">
+        <v>103213.82</v>
+      </c>
+      <c r="I9" s="17" t="n">
+        <v>256998.27</v>
       </c>
     </row>
     <row r="10">
@@ -2750,45 +2791,45 @@
           <t>Lücke zum Selbstkostenpreis</t>
         </is>
       </c>
-      <c r="B10" s="16" t="n">
-        <v>103404.09</v>
-      </c>
-      <c r="C10" s="16" t="n">
-        <v>14953.75</v>
-      </c>
-      <c r="E10" s="16" t="n">
-        <v>85571.36</v>
-      </c>
-      <c r="F10" s="16" t="n">
-        <v>5046.22</v>
-      </c>
-      <c r="H10" s="16" t="n">
-        <v>81166.25</v>
-      </c>
-      <c r="I10" s="16" t="n">
-        <v>1322.91</v>
+      <c r="B10" s="17" t="n">
+        <v>103222.86</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>69488.28999999999</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>83380.96000000001</v>
+      </c>
+      <c r="F10" s="17" t="n">
+        <v>96345.05</v>
+      </c>
+      <c r="H10" s="17" t="n">
+        <v>39539.75</v>
+      </c>
+      <c r="I10" s="17" t="n">
+        <v>90238.03</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Haus als Ganzes mit einem Kredit</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr"/>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr"/>
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>A: 340 m²</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>B: 540 m²</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>B (Haupt): 540 m²</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
         <is>
           <t>C: 540 m², 3 Vollgeschosse + Holz-Penthouse</t>
         </is>
@@ -2800,14 +2841,14 @@
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B15" s="16" t="n">
+      <c r="B15" s="17" t="n">
         <v>2716271</v>
       </c>
-      <c r="C15" s="16" t="n">
-        <v>4112256</v>
-      </c>
-      <c r="D15" s="16" t="n">
-        <v>5478456</v>
+      <c r="C15" s="17" t="n">
+        <v>4108116</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <v>5474316</v>
       </c>
     </row>
     <row r="16">
@@ -2816,14 +2857,14 @@
           <t>Rate pro Monat</t>
         </is>
       </c>
-      <c r="B16" s="16" t="n">
+      <c r="B16" s="17" t="n">
         <v>10345.03</v>
       </c>
-      <c r="C16" s="16" t="n">
-        <v>15654.96</v>
-      </c>
-      <c r="D16" s="16" t="n">
-        <v>20851.61</v>
+      <c r="C16" s="17" t="n">
+        <v>15639.22</v>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>20835.86</v>
       </c>
     </row>
     <row r="17">
@@ -2832,14 +2873,14 @@
           <t>Ergebnis pro Monat bei 50.000 € Umsatz</t>
         </is>
       </c>
-      <c r="B17" s="21" t="n">
+      <c r="B17" s="22" t="n">
         <v>9686.969999999999</v>
       </c>
-      <c r="C17" s="21" t="n">
-        <v>7889.68</v>
-      </c>
-      <c r="D17" s="21" t="n">
-        <v>6867.45</v>
+      <c r="C17" s="22" t="n">
+        <v>7905.43</v>
+      </c>
+      <c r="D17" s="22" t="n">
+        <v>6883.2</v>
       </c>
     </row>
     <row r="18">
@@ -2848,58 +2889,58 @@
           <t>Break-even Gastro-Umsatz</t>
         </is>
       </c>
-      <c r="B18" s="16" t="n">
+      <c r="B18" s="17" t="n">
         <v>18239.43</v>
       </c>
-      <c r="C18" s="16" t="n">
-        <v>24132.19</v>
-      </c>
-      <c r="D18" s="16" t="n">
-        <v>27483.77</v>
+      <c r="C18" s="17" t="n">
+        <v>24080.56</v>
+      </c>
+      <c r="D18" s="17" t="n">
+        <v>27432.14</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>B: EG 540 m² (Gastro 290 + Büro 150), 1. OG 540 m², Staffel 420 m² mit 120 m² Terrasse. C: zusätzlich 2. OG 540 m², Höhe ca. 13 m. Nur mit Ausnahme der Stadt (Baufenster, II Vollgeschosse, 12 m).</t>
+          <t>B (Hauptvariante): EG 540 m² (Gastro 290 + Büro 150), 1. OG 540 m², Staffel 460 m² mit 72 m² Terrasse. C: zusätzlich 2. OG 540 m², Höhe ca. 13 m. Nur mit Ausnahme der Stadt (Baufenster, II Vollgeschosse, 12 m).</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="inlineStr">
-        <is>
-          <t>Ziel: 250 € Plus je Wohnung (Käufer ohne Eigenkapital, ohne Tilgung, Variante A)</t>
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Ziel: 250 € Plus je Wohnung (Käufer ohne Eigenkapital, ohne Tilgung, Variante B)</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="inlineStr"/>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>1. OG 85 m²</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="inlineStr">
-        <is>
-          <t>Staffel 63 m²</t>
-        </is>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="A23" s="12" t="inlineStr"/>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>1. OG 83 m²</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>Staffel 103 m²</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Du</t>
         </is>
       </c>
-      <c r="E23" s="12" t="inlineStr">
+      <c r="E23" s="13" t="inlineStr">
         <is>
           <t>Zins 4,0 %: 1. OG</t>
         </is>
       </c>
-      <c r="F23" s="12" t="inlineStr">
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>Zins 4,0 %: Staffel</t>
         </is>
       </c>
-      <c r="G23" s="12" t="inlineStr">
+      <c r="G23" s="13" t="inlineStr">
         <is>
           <t>Zins 4,0 %: Du</t>
         </is>
@@ -2911,17 +2952,17 @@
           <t>Verkaufspreis</t>
         </is>
       </c>
-      <c r="B24" s="16" t="n">
-        <v>206991</v>
-      </c>
-      <c r="C24" s="16" t="n">
-        <v>206991</v>
-      </c>
-      <c r="E24" s="16" t="n">
-        <v>168818</v>
-      </c>
-      <c r="F24" s="16" t="n">
-        <v>168818</v>
+      <c r="B24" s="17" t="n">
+        <v>200194</v>
+      </c>
+      <c r="C24" s="17" t="n">
+        <v>270200</v>
+      </c>
+      <c r="E24" s="17" t="n">
+        <v>163297</v>
+      </c>
+      <c r="F24" s="17" t="n">
+        <v>220400</v>
       </c>
     </row>
     <row r="25">
@@ -2930,17 +2971,17 @@
           <t>Selbstkosten</t>
         </is>
       </c>
-      <c r="B25" s="16" t="n">
-        <v>314624.67</v>
-      </c>
-      <c r="C25" s="16" t="n">
-        <v>226174.33</v>
-      </c>
-      <c r="E25" s="16" t="n">
-        <v>314624.67</v>
-      </c>
-      <c r="F25" s="16" t="n">
-        <v>226174.33</v>
+      <c r="B25" s="17" t="n">
+        <v>289808.6</v>
+      </c>
+      <c r="C25" s="17" t="n">
+        <v>353343.32</v>
+      </c>
+      <c r="E25" s="17" t="n">
+        <v>289808.6</v>
+      </c>
+      <c r="F25" s="17" t="n">
+        <v>353343.32</v>
       </c>
     </row>
     <row r="26">
@@ -2949,23 +2990,23 @@
           <t>Nachlass (von dir getragen)</t>
         </is>
       </c>
-      <c r="B26" s="16" t="n">
-        <v>107633.67</v>
-      </c>
-      <c r="C26" s="16" t="n">
-        <v>19183.33</v>
-      </c>
-      <c r="D26" s="16" t="n">
-        <v>380451</v>
-      </c>
-      <c r="E26" s="16" t="n">
-        <v>145806.67</v>
-      </c>
-      <c r="F26" s="16" t="n">
-        <v>57356.33</v>
-      </c>
-      <c r="G26" s="16" t="n">
-        <v>609489</v>
+      <c r="B26" s="17" t="n">
+        <v>89614.60000000001</v>
+      </c>
+      <c r="C26" s="17" t="n">
+        <v>83143.32000000001</v>
+      </c>
+      <c r="D26" s="17" t="n">
+        <v>697502.99</v>
+      </c>
+      <c r="E26" s="17" t="n">
+        <v>126511.6</v>
+      </c>
+      <c r="F26" s="17" t="n">
+        <v>132943.32</v>
+      </c>
+      <c r="G26" s="17" t="n">
+        <v>1031387.99</v>
       </c>
     </row>
     <row r="27">
@@ -2974,23 +3015,23 @@
           <t>Rate pro Monat</t>
         </is>
       </c>
-      <c r="B27" s="16" t="n">
-        <v>605</v>
-      </c>
-      <c r="C27" s="16" t="n">
-        <v>605</v>
-      </c>
-      <c r="D27" s="16" t="n">
-        <v>5278.06</v>
-      </c>
-      <c r="E27" s="16" t="n">
-        <v>605</v>
-      </c>
-      <c r="F27" s="16" t="n">
-        <v>605</v>
-      </c>
-      <c r="G27" s="16" t="n">
-        <v>7084.47</v>
+      <c r="B27" s="17" t="n">
+        <v>584.88</v>
+      </c>
+      <c r="C27" s="17" t="n">
+        <v>789.41</v>
+      </c>
+      <c r="D27" s="17" t="n">
+        <v>8125.22</v>
+      </c>
+      <c r="E27" s="17" t="n">
+        <v>584.88</v>
+      </c>
+      <c r="F27" s="17" t="n">
+        <v>789.41</v>
+      </c>
+      <c r="G27" s="17" t="n">
+        <v>10853.29</v>
       </c>
     </row>
     <row r="28">
@@ -2999,74 +3040,74 @@
           <t>Ergebnis pro Monat</t>
         </is>
       </c>
-      <c r="B28" s="21" t="n">
+      <c r="B28" s="22" t="n">
         <v>250</v>
       </c>
-      <c r="C28" s="21" t="n">
+      <c r="C28" s="22" t="n">
         <v>250</v>
       </c>
-      <c r="D28" s="21" t="n">
-        <v>9971.940000000001</v>
-      </c>
-      <c r="E28" s="21" t="n">
+      <c r="D28" s="22" t="n">
+        <v>7124.78</v>
+      </c>
+      <c r="E28" s="22" t="n">
         <v>250</v>
       </c>
-      <c r="F28" s="21" t="n">
+      <c r="F28" s="22" t="n">
         <v>250</v>
       </c>
-      <c r="G28" s="21" t="n">
-        <v>8165.53</v>
+      <c r="G28" s="22" t="n">
+        <v>4396.71</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="14" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>Verkaufsplan (Vorschlag), ohne Förderung, 2.200 €/m², tilgungsfrei, 3,3 % Zins, Notar 2 %, Grunderwerbsteuer 5 % (Vater frei)</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>Partei</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
+      <c r="B32" s="13" t="inlineStr">
         <is>
           <t>Wohnung</t>
         </is>
       </c>
-      <c r="C32" s="12" t="inlineStr">
+      <c r="C32" s="13" t="inlineStr">
         <is>
           <t>Verkaufspreis</t>
         </is>
       </c>
-      <c r="D32" s="12" t="inlineStr">
+      <c r="D32" s="13" t="inlineStr">
         <is>
           <t>Selbstkosten</t>
         </is>
       </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="E32" s="13" t="inlineStr">
         <is>
           <t>Differenz (von dir getragen)</t>
         </is>
       </c>
-      <c r="F32" s="12" t="inlineStr">
+      <c r="F32" s="13" t="inlineStr">
         <is>
           <t>Notar, Steuer</t>
         </is>
       </c>
-      <c r="G32" s="12" t="inlineStr">
+      <c r="G32" s="13" t="inlineStr">
         <is>
           <t>Rate (nur Zinsen)</t>
         </is>
       </c>
-      <c r="H32" s="12" t="inlineStr">
+      <c r="H32" s="13" t="inlineStr">
         <is>
           <t>Ergebnis pro Monat</t>
         </is>
       </c>
-      <c r="I32" s="12" t="inlineStr">
+      <c r="I32" s="13" t="inlineStr">
         <is>
           <t>Ergebnis zum Selbstkostenpreis</t>
         </is>
@@ -3080,29 +3121,29 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>1. OG, 85 m²</t>
-        </is>
-      </c>
-      <c r="C33" s="16" t="n">
-        <v>253246.09</v>
-      </c>
-      <c r="D33" s="16" t="n">
-        <v>314624.67</v>
-      </c>
-      <c r="E33" s="16" t="n">
-        <v>61378.58</v>
-      </c>
-      <c r="F33" s="16" t="n">
-        <v>5064.92</v>
-      </c>
-      <c r="G33" s="16" t="n">
-        <v>755</v>
-      </c>
-      <c r="H33" s="21" t="n">
+          <t>1. OG, 83 m²</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="n">
+        <v>246603.85</v>
+      </c>
+      <c r="D33" s="17" t="n">
+        <v>289808.6</v>
+      </c>
+      <c r="E33" s="17" t="n">
+        <v>43204.76</v>
+      </c>
+      <c r="F33" s="17" t="n">
+        <v>4932.08</v>
+      </c>
+      <c r="G33" s="17" t="n">
+        <v>734.88</v>
+      </c>
+      <c r="H33" s="22" t="n">
         <v>100</v>
       </c>
-      <c r="I33" s="21" t="n">
-        <v>-82.98999999999999</v>
+      <c r="I33" s="22" t="n">
+        <v>-28.75</v>
       </c>
     </row>
     <row r="34">
@@ -3113,191 +3154,257 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>1. OG, 85 m²</t>
-        </is>
-      </c>
-      <c r="C34" s="16" t="n">
-        <v>241412.16</v>
-      </c>
-      <c r="D34" s="16" t="n">
-        <v>314624.67</v>
-      </c>
-      <c r="E34" s="16" t="n">
-        <v>73212.50999999999</v>
-      </c>
-      <c r="F34" s="16" t="n">
-        <v>16898.85</v>
-      </c>
-      <c r="G34" s="16" t="n">
-        <v>755</v>
-      </c>
-      <c r="H34" s="21" t="n">
+          <t>1. OG, 83 m²</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="n">
+        <v>235080.3</v>
+      </c>
+      <c r="D34" s="17" t="n">
+        <v>289808.6</v>
+      </c>
+      <c r="E34" s="17" t="n">
+        <v>54728.3</v>
+      </c>
+      <c r="F34" s="17" t="n">
+        <v>16455.62</v>
+      </c>
+      <c r="G34" s="17" t="n">
+        <v>734.88</v>
+      </c>
+      <c r="H34" s="22" t="n">
         <v>100</v>
       </c>
-      <c r="I34" s="21" t="n">
-        <v>-128.97</v>
+      <c r="I34" s="22" t="n">
+        <v>-71.09</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Du (eigene Wohnung)</t>
+          <t>Du (Wohnung 1, eigene)</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>1. OG, 85 m²</t>
-        </is>
-      </c>
-      <c r="C35" s="16" t="n">
-        <v>314624.67</v>
-      </c>
-      <c r="D35" s="16" t="n">
-        <v>314624.67</v>
-      </c>
-      <c r="E35" s="16" t="n">
+          <t>1. OG, 83 m²</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="n">
+        <v>289808.6</v>
+      </c>
+      <c r="D35" s="17" t="n">
+        <v>289808.6</v>
+      </c>
+      <c r="E35" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="F35" s="16" t="n">
+      <c r="F35" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="G35" s="16" t="n">
-        <v>919.6</v>
-      </c>
-      <c r="H35" s="21" t="n">
-        <v>-64.59999999999999</v>
-      </c>
-      <c r="I35" s="21" t="n">
-        <v>-64.59999999999999</v>
+      <c r="G35" s="17" t="n">
+        <v>846.7</v>
+      </c>
+      <c r="H35" s="22" t="n">
+        <v>-11.82</v>
+      </c>
+      <c r="I35" s="22" t="n">
+        <v>-11.82</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Onkel 1</t>
+          <t>Du (Wohnung 2, vermietet)</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Staffel, 63 m²</t>
-        </is>
-      </c>
-      <c r="C36" s="16" t="n">
-        <v>226174.33</v>
-      </c>
-      <c r="D36" s="16" t="n">
-        <v>226174.33</v>
-      </c>
-      <c r="E36" s="16" t="n">
+          <t>1. OG, 83 m²</t>
+        </is>
+      </c>
+      <c r="C36" s="17" t="n">
+        <v>289808.6</v>
+      </c>
+      <c r="D36" s="17" t="n">
+        <v>289808.6</v>
+      </c>
+      <c r="E36" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="F36" s="16" t="n">
-        <v>15832.2</v>
-      </c>
-      <c r="G36" s="16" t="n">
-        <v>707.34</v>
-      </c>
-      <c r="H36" s="21" t="n">
-        <v>147.66</v>
-      </c>
-      <c r="I36" s="21" t="n">
-        <v>147.66</v>
+      <c r="F36" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="17" t="n">
+        <v>846.7</v>
+      </c>
+      <c r="H36" s="22" t="n">
+        <v>-11.82</v>
+      </c>
+      <c r="I36" s="22" t="n">
+        <v>-11.82</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Onkel 2</t>
+          <t>Du (Wohnung 3, vermietet)</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Staffel, 63 m²</t>
-        </is>
-      </c>
-      <c r="C37" s="16" t="n">
-        <v>226174.33</v>
-      </c>
-      <c r="D37" s="16" t="n">
-        <v>226174.33</v>
-      </c>
-      <c r="E37" s="16" t="n">
+          <t>1. OG, 83 m²</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="n">
+        <v>289808.6</v>
+      </c>
+      <c r="D37" s="17" t="n">
+        <v>289808.6</v>
+      </c>
+      <c r="E37" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="F37" s="16" t="n">
-        <v>15832.2</v>
-      </c>
-      <c r="G37" s="16" t="n">
-        <v>707.34</v>
-      </c>
-      <c r="H37" s="21" t="n">
-        <v>147.66</v>
-      </c>
-      <c r="I37" s="21" t="n">
-        <v>147.66</v>
+      <c r="F37" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="17" t="n">
+        <v>846.7</v>
+      </c>
+      <c r="H37" s="22" t="n">
+        <v>-11.82</v>
+      </c>
+      <c r="I37" s="22" t="n">
+        <v>-11.82</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>Onkel 3</t>
+          <t>Onkel 1</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Staffel, 63 m²</t>
-        </is>
-      </c>
-      <c r="C38" s="16" t="n">
-        <v>226174.33</v>
-      </c>
-      <c r="D38" s="16" t="n">
-        <v>226174.33</v>
-      </c>
-      <c r="E38" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" s="16" t="n">
-        <v>15832.2</v>
-      </c>
-      <c r="G38" s="16" t="n">
-        <v>707.34</v>
-      </c>
-      <c r="H38" s="21" t="n">
-        <v>147.66</v>
-      </c>
-      <c r="I38" s="21" t="n">
-        <v>147.66</v>
+          <t>Staffel, 103 m²</t>
+        </is>
+      </c>
+      <c r="C38" s="17" t="n">
+        <v>300506.88</v>
+      </c>
+      <c r="D38" s="17" t="n">
+        <v>353343.32</v>
+      </c>
+      <c r="E38" s="17" t="n">
+        <v>52836.45</v>
+      </c>
+      <c r="F38" s="17" t="n">
+        <v>21035.48</v>
+      </c>
+      <c r="G38" s="17" t="n">
+        <v>939.41</v>
+      </c>
+      <c r="H38" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="I38" s="22" t="n">
+        <v>-65.17</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Onkel 2</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Staffel, 103 m²</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="n">
+        <v>300506.88</v>
+      </c>
+      <c r="D39" s="17" t="n">
+        <v>353343.32</v>
+      </c>
+      <c r="E39" s="17" t="n">
+        <v>52836.45</v>
+      </c>
+      <c r="F39" s="17" t="n">
+        <v>21035.48</v>
+      </c>
+      <c r="G39" s="17" t="n">
+        <v>939.41</v>
+      </c>
+      <c r="H39" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="I39" s="22" t="n">
+        <v>-65.17</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
+          <t>Onkel 3</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Staffel, 103 m²</t>
+        </is>
+      </c>
+      <c r="C40" s="17" t="n">
+        <v>300506.88</v>
+      </c>
+      <c r="D40" s="17" t="n">
+        <v>353343.32</v>
+      </c>
+      <c r="E40" s="17" t="n">
+        <v>52836.45</v>
+      </c>
+      <c r="F40" s="17" t="n">
+        <v>21035.48</v>
+      </c>
+      <c r="G40" s="17" t="n">
+        <v>939.41</v>
+      </c>
+      <c r="H40" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="I40" s="22" t="n">
+        <v>-65.17</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
           <t>Differenz gesamt (von dir getragen)</t>
         </is>
       </c>
-      <c r="C40" s="16" t="n">
-        <v>134591.08</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="C42" s="17" t="n">
+        <v>256442.4</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>Zinsen auf die Differenz pro Monat</t>
         </is>
       </c>
-      <c r="C41" s="16" t="n">
-        <v>393.39</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="14" t="inlineStr">
-        <is>
-          <t>Dein Ergebnis pro Monat (Gastro − Rate EG − Zinsen Differenz + eigene Wohnung)</t>
-        </is>
-      </c>
-      <c r="C42" s="21" t="n">
-        <v>10625.95</v>
+      <c r="C43" s="17" t="n">
+        <v>749.22</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t>Dein Ergebnis pro Monat (Gastro − Rate EG − Zinsen Differenz + deine drei Wohnungen)</t>
+        </is>
+      </c>
+      <c r="C44" s="22" t="n">
+        <v>8377.92</v>
       </c>
     </row>
   </sheetData>
@@ -3322,7 +3429,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Variante: Mittelgeschoss doppelt (4 Ebenen)</t>
+          <t>Variante: Mittelgeschoss doppelt (4 Ebenen, Basis Variante A)</t>
         </is>
       </c>
     </row>
@@ -3334,13 +3441,13 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr"/>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr"/>
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>3 Ebenen</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>4 Ebenen</t>
         </is>
@@ -3352,10 +3459,10 @@
           <t>Wohnungen</t>
         </is>
       </c>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="23" t="n">
         <v>6</v>
       </c>
-      <c r="C5" s="22" t="n">
+      <c r="C5" s="23" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3365,10 +3472,10 @@
           <t>BGF (m²)</t>
         </is>
       </c>
-      <c r="B6" s="23" t="n">
+      <c r="B6" s="24" t="n">
         <v>960</v>
       </c>
-      <c r="C6" s="23" t="n">
+      <c r="C6" s="24" t="n">
         <v>1300</v>
       </c>
     </row>
@@ -3378,10 +3485,10 @@
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="17" t="n">
         <v>2716271</v>
       </c>
-      <c r="C7" s="16" t="n">
+      <c r="C7" s="17" t="n">
         <v>3576471</v>
       </c>
     </row>
@@ -3391,10 +3498,10 @@
           <t>Rate (Plan)</t>
         </is>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="B8" s="17" t="n">
         <v>10345.03</v>
       </c>
-      <c r="C8" s="16" t="n">
+      <c r="C8" s="17" t="n">
         <v>13616.99</v>
       </c>
     </row>
@@ -3404,10 +3511,10 @@
           <t>Ergebnis pro Monat ohne Förderung</t>
         </is>
       </c>
-      <c r="B9" s="21" t="n">
+      <c r="B9" s="22" t="n">
         <v>9686.969999999999</v>
       </c>
-      <c r="C9" s="21" t="n">
+      <c r="C9" s="22" t="n">
         <v>8980.01</v>
       </c>
     </row>
@@ -3417,10 +3524,10 @@
           <t>Ergebnis pro Monat mit 15 % Förderung</t>
         </is>
       </c>
-      <c r="B10" s="21" t="n">
+      <c r="B10" s="22" t="n">
         <v>11238.73</v>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C10" s="22" t="n">
         <v>11022.56</v>
       </c>
     </row>
@@ -3465,7 +3572,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>• Miete 950 € je Wohnung liegt über den Portalwerten für Neubau in Werlte (ca. 10,70–11,02 €/m²).</t>
+          <t>• Miete 11,18 €/m² (950 € für 85 m²) liegt am oberen Rand der Portalwerte für Neubau in Werlte (ca. 10,70–11,02 €/m²).</t>
         </is>
       </c>
     </row>
@@ -3486,7 +3593,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>• Staffelgeschoss (ca. 280 m², Holzbau, schmale Terrasse rundum) und Gesamthöhe ca. 9,90 m müssen mit der Stadt abgestimmt werden.</t>
+          <t>• Grundfläche 540 m² (Baufenster im Plan geschätzt kleiner), Staffelgeschoss (ca. 460 m², Holzbau, schmale Terrasse rundum) und Gesamthöhe ca. 9,90 m müssen mit der Stadt abgestimmt werden.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gastro im ganzen EG (460 m²), Gastro-Konzept-Präsentation, neue Gastro- und Außenbilder
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJGZfxHv7bzYyqdLwg8aFJ
</commit_message>
<xml_diff>
--- a/praesentation/Rechenmodell_Baufeld3.xlsx
+++ b/praesentation/Rechenmodell_Baufeld3.xlsx
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>290</v>
+        <v>460</v>
       </c>
       <c r="C27" s="2" t="inlineStr"/>
     </row>
@@ -1010,11 +1010,11 @@
         </is>
       </c>
       <c r="B42" s="6" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>vermietet</t>
+          <t>in Variante B kein Büro, Gastro nutzt das ganze EG</t>
         </is>
       </c>
     </row>
@@ -2272,19 +2272,19 @@
         <v>15639.22</v>
       </c>
       <c r="D5" s="22" t="n">
-        <v>7905.43</v>
+        <v>6351.43</v>
       </c>
       <c r="E5" s="17" t="n">
         <v>18392.63</v>
       </c>
       <c r="F5" s="22" t="n">
-        <v>5152.01</v>
+        <v>3598.01</v>
       </c>
       <c r="G5" s="17" t="n">
-        <v>24080.56</v>
+        <v>29175.64</v>
       </c>
       <c r="H5" s="17" t="n">
-        <v>33108.15</v>
+        <v>38203.23</v>
       </c>
     </row>
     <row r="6">
@@ -2298,19 +2298,19 @@
         <v>14857.26</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>8687.389999999999</v>
+        <v>7133.39</v>
       </c>
       <c r="E6" s="17" t="n">
         <v>17473</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>6071.65</v>
+        <v>4517.65</v>
       </c>
       <c r="G6" s="17" t="n">
-        <v>21516.75</v>
+        <v>26611.83</v>
       </c>
       <c r="H6" s="17" t="n">
-        <v>30092.97</v>
+        <v>35188.05</v>
       </c>
     </row>
     <row r="7">
@@ -2324,19 +2324,19 @@
         <v>14075.3</v>
       </c>
       <c r="D7" s="22" t="n">
-        <v>9469.35</v>
+        <v>7915.35</v>
       </c>
       <c r="E7" s="17" t="n">
         <v>16553.37</v>
       </c>
       <c r="F7" s="22" t="n">
-        <v>6991.28</v>
+        <v>5437.28</v>
       </c>
       <c r="G7" s="17" t="n">
-        <v>18952.95</v>
+        <v>24048.03</v>
       </c>
       <c r="H7" s="17" t="n">
-        <v>27077.78</v>
+        <v>32172.86</v>
       </c>
     </row>
     <row r="8">
@@ -2350,19 +2350,19 @@
         <v>13293.33</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>10251.31</v>
+        <v>8697.309999999999</v>
       </c>
       <c r="E8" s="17" t="n">
         <v>15633.74</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>7910.91</v>
+        <v>6356.91</v>
       </c>
       <c r="G8" s="17" t="n">
-        <v>16389.14</v>
+        <v>21484.22</v>
       </c>
       <c r="H8" s="17" t="n">
-        <v>24062.6</v>
+        <v>29157.68</v>
       </c>
     </row>
     <row r="9">
@@ -2376,19 +2376,19 @@
         <v>12511.37</v>
       </c>
       <c r="D9" s="22" t="n">
-        <v>11033.27</v>
+        <v>9479.27</v>
       </c>
       <c r="E9" s="17" t="n">
         <v>14714.11</v>
       </c>
       <c r="F9" s="22" t="n">
-        <v>8830.540000000001</v>
+        <v>7276.54</v>
       </c>
       <c r="G9" s="17" t="n">
-        <v>13825.33</v>
+        <v>18920.42</v>
       </c>
       <c r="H9" s="17" t="n">
-        <v>21047.41</v>
+        <v>26142.49</v>
       </c>
     </row>
     <row r="10">
@@ -2402,19 +2402,19 @@
         <v>11729.41</v>
       </c>
       <c r="D10" s="22" t="n">
-        <v>11815.23</v>
+        <v>10261.23</v>
       </c>
       <c r="E10" s="17" t="n">
         <v>13794.48</v>
       </c>
       <c r="F10" s="22" t="n">
-        <v>9750.17</v>
+        <v>8196.17</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>11261.53</v>
+        <v>16356.61</v>
       </c>
       <c r="H10" s="17" t="n">
-        <v>18032.22</v>
+        <v>23127.31</v>
       </c>
     </row>
     <row r="12">
@@ -2461,19 +2461,19 @@
         <v>0</v>
       </c>
       <c r="B14" s="22" t="n">
-        <v>4855.43</v>
+        <v>3301.43</v>
       </c>
       <c r="C14" s="22" t="n">
-        <v>6380.43</v>
+        <v>4826.43</v>
       </c>
       <c r="D14" s="22" t="n">
-        <v>7905.43</v>
+        <v>6351.43</v>
       </c>
       <c r="E14" s="22" t="n">
-        <v>9430.43</v>
+        <v>7876.43</v>
       </c>
       <c r="F14" s="22" t="n">
-        <v>10955.43</v>
+        <v>9401.43</v>
       </c>
     </row>
     <row r="15">
@@ -2481,19 +2481,19 @@
         <v>0.1</v>
       </c>
       <c r="B15" s="22" t="n">
-        <v>6419.35</v>
+        <v>4865.35</v>
       </c>
       <c r="C15" s="22" t="n">
-        <v>7944.35</v>
+        <v>6390.35</v>
       </c>
       <c r="D15" s="22" t="n">
-        <v>9469.35</v>
+        <v>7915.35</v>
       </c>
       <c r="E15" s="22" t="n">
-        <v>10994.35</v>
+        <v>9440.35</v>
       </c>
       <c r="F15" s="22" t="n">
-        <v>12519.35</v>
+        <v>10965.35</v>
       </c>
     </row>
     <row r="16">
@@ -2501,19 +2501,19 @@
         <v>0.15</v>
       </c>
       <c r="B16" s="22" t="n">
-        <v>7201.31</v>
+        <v>5647.31</v>
       </c>
       <c r="C16" s="22" t="n">
-        <v>8726.309999999999</v>
+        <v>7172.31</v>
       </c>
       <c r="D16" s="22" t="n">
-        <v>10251.31</v>
+        <v>8697.309999999999</v>
       </c>
       <c r="E16" s="22" t="n">
-        <v>11776.31</v>
+        <v>10222.31</v>
       </c>
       <c r="F16" s="22" t="n">
-        <v>13301.31</v>
+        <v>11747.31</v>
       </c>
     </row>
     <row r="17">
@@ -2521,19 +2521,19 @@
         <v>0.2</v>
       </c>
       <c r="B17" s="22" t="n">
-        <v>7983.27</v>
+        <v>6429.27</v>
       </c>
       <c r="C17" s="22" t="n">
-        <v>9508.27</v>
+        <v>7954.27</v>
       </c>
       <c r="D17" s="22" t="n">
-        <v>11033.27</v>
+        <v>9479.27</v>
       </c>
       <c r="E17" s="22" t="n">
-        <v>12558.27</v>
+        <v>11004.27</v>
       </c>
       <c r="F17" s="22" t="n">
-        <v>14083.27</v>
+        <v>12529.27</v>
       </c>
     </row>
   </sheetData>
@@ -2605,7 +2605,7 @@
       </c>
       <c r="G4" s="13" t="inlineStr">
         <is>
-          <t>B: Gastro + Büro (Du)</t>
+          <t>B: Gastro (Du)</t>
         </is>
       </c>
       <c r="H4" s="13" t="inlineStr">
@@ -2714,7 +2714,7 @@
         <v>1039.41</v>
       </c>
       <c r="G7" s="17" t="n">
-        <v>16600</v>
+        <v>15250</v>
       </c>
       <c r="H7" s="17" t="n">
         <v>417.44</v>
@@ -2723,7 +2723,7 @@
         <v>1039.41</v>
       </c>
       <c r="J7" s="17" t="n">
-        <v>16600</v>
+        <v>15250</v>
       </c>
     </row>
     <row r="8">
@@ -2748,7 +2748,7 @@
         <v>-305.73</v>
       </c>
       <c r="G8" s="22" t="n">
-        <v>10512.59</v>
+        <v>9162.59</v>
       </c>
       <c r="H8" s="22" t="n">
         <v>-126.01</v>
@@ -2757,7 +2757,7 @@
         <v>-282.48</v>
       </c>
       <c r="J8" s="22" t="n">
-        <v>10594.47</v>
+        <v>9244.469999999999</v>
       </c>
     </row>
     <row r="9">
@@ -2877,10 +2877,10 @@
         <v>9686.969999999999</v>
       </c>
       <c r="C17" s="22" t="n">
-        <v>7905.43</v>
+        <v>6351.43</v>
       </c>
       <c r="D17" s="22" t="n">
-        <v>6883.2</v>
+        <v>5329.2</v>
       </c>
     </row>
     <row r="18">
@@ -2893,16 +2893,16 @@
         <v>18239.43</v>
       </c>
       <c r="C18" s="17" t="n">
-        <v>24080.56</v>
+        <v>29175.64</v>
       </c>
       <c r="D18" s="17" t="n">
-        <v>27432.14</v>
+        <v>32527.22</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>B (Hauptvariante): EG 540 m² (Gastro 290 + Büro 150), 1. OG 540 m², Staffel 460 m² mit 72 m² Terrasse. C: zusätzlich 2. OG 540 m², Höhe ca. 13 m. Nur mit Ausnahme der Stadt (Baufenster, II Vollgeschosse, 12 m).</t>
+          <t>B (Hauptvariante): EG 540 m² (Gastro 460), 1. OG 540 m², Staffel 460 m² mit 72 m² Terrasse. C: zusätzlich 2. OG 540 m², Höhe ca. 13 m. Nur mit Ausnahme der Stadt (Baufenster, II Vollgeschosse, 12 m).</t>
         </is>
       </c>
     </row>

</xml_diff>